<commit_message>
Align BSCR workings labels with templates
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -31160,7 +31160,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CATASTROPHE RISK RETURN: EP CURVE TOTAL INPUTS</t>
+          <t>CATASTROPHE RISK RETURN: EP CURVE TOTAL (TABLE 15)</t>
         </is>
       </c>
     </row>
@@ -31174,17 +31174,17 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Required input</t>
+          <t>Loss Return period (years)</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Gross</t>
+          <t>Gross loss</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Net</t>
+          <t>Net loss</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -31280,7 +31280,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Property catastrophe premium</t>
+          <t>Total statutory property catastrophe premium modelled</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -31292,7 +31292,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>All other catastrophe premium</t>
+          <t>Total all other catastrophe premium modelled</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -31339,7 +31339,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CATASTROPHE RISK RETURN: EP CURVE INSURANCE INPUTS</t>
+          <t>CATASTROPHE RISK RETURN: EP CURVE INSURANCE (TABLE 15A)</t>
         </is>
       </c>
     </row>
@@ -31353,17 +31353,17 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Required input</t>
+          <t>Loss Return period (years)</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Gross</t>
+          <t>Gross loss</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Net</t>
+          <t>Net loss</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -31459,7 +31459,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Property catastrophe premium</t>
+          <t>Total statutory property catastrophe premium modelled</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -31471,7 +31471,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>All other catastrophe premium</t>
+          <t>Total all other catastrophe premium modelled</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -31518,7 +31518,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CATASTROPHE RISK RETURN: REGIONS-PERILS INPUTS</t>
+          <t>CATASTROPHE RISK RETURN: EXCEEDANCE PROBABILITY  (EP) CURVE  FOR REGIONS-PERILS (TABLE 15B)</t>
         </is>
       </c>
     </row>
@@ -31532,7 +31532,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Region</t>
+          <t>Exposure</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -31554,7 +31554,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Atlantic Basin Hurricane</t>
+          <t>Exposure to Atlantic Basin Hurricane</t>
         </is>
       </c>
       <c r="B4" s="7">
@@ -31574,7 +31574,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>North American Earthquake</t>
+          <t>Exposure to North American Earthquake</t>
         </is>
       </c>
       <c r="B5" s="7">
@@ -31594,7 +31594,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>European Windstorm</t>
+          <t>Exposure to European Windstorm</t>
         </is>
       </c>
       <c r="B6" s="7">
@@ -31614,7 +31614,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Japanese Earthquake</t>
+          <t>Exposure to Japanese Earthquake</t>
         </is>
       </c>
       <c r="B7" s="7">
@@ -31634,7 +31634,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Japanese Typhoon</t>
+          <t>Exposure to Japanese Typhoon</t>
         </is>
       </c>
       <c r="B8" s="7">
@@ -31654,7 +31654,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Premium inputs</t>
+          <t>Total statutory property catastrophe premium</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -31666,7 +31666,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EP curve loss inputs</t>
+          <t>Exceedance probability information:</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -31697,7 +31697,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CATASTROPHE RISK RETURN: DATA ANALYSIS INPUTS</t>
+          <t>CATASTROPHE RISK RETURN: DATA  ANALYSIS (TABLE 15E)</t>
         </is>
       </c>
     </row>
@@ -31711,7 +31711,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Contract classification</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -31753,7 +31753,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>All contracts - geographic split only</t>
+          <t>All contracts - all exposures</t>
         </is>
       </c>
       <c r="B4" s="7">
@@ -31789,7 +31789,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Modelled</t>
+          <t>modellable</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -31801,7 +31801,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Not modelled</t>
+          <t>Not modellable</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -31813,7 +31813,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Control: HIC total output</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="B8" s="7">

</xml_diff>

<commit_message>
Clarify BSCR workbook processing tabs
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -13,9 +13,9 @@
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="3" xr2:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
   </bookViews>
   <sheets>
-    <sheet name="piv" sheetId="2" r:id="rId1"/>
-    <sheet name="output" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
+    <sheet name="BSCR Pivot Summary" sheetId="2" r:id="rId1"/>
+    <sheet name="BSCR Output" sheetId="1" r:id="rId2"/>
+    <sheet name="BSCR Source Data" sheetId="3" r:id="rId3"/>
     <sheet name="AUDIT_SUMMARY" sheetId="4" r:id="rId10"/>
     <sheet name="Settings" sheetId="5" r:id="rId11"/>
     <sheet name="Schedule X(a)" sheetId="6" r:id="rId12"/>
@@ -24,8 +24,8 @@
     <sheet name="Schedule X(f)" sheetId="9" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">output!$A$1:$F$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BSCR Output'!$A$1:$F$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BSCR Source Data'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
   <pivotCaches>
@@ -1189,7 +1189,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" refreshOnLoad="1" mc:Ignorable="xr" r:id="rId1" refreshedBy="Richard Hampton" refreshedDate="46090.700917708331" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="49" xr:uid="{B1A2DC09-0005-4103-9A04-052000D9B748}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:J50" sheet="output"/>
+    <worksheetSource ref="A1:J50" sheet="BSCR Output"/>
   </cacheSource>
   <cacheFields count="10">
     <cacheField name="bscr_entity" numFmtId="0">
@@ -1297,7 +1297,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" refreshOnLoad="1" mc:Ignorable="xr" r:id="rId1" refreshedBy="Faye Williams" refreshedDate="46106.622011574073" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="453" xr:uid="{8B38D0A1-59CD-453E-BBD5-7D49D4105093}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:K1048576" sheet="Sheet1"/>
+    <worksheetSource ref="A1:K1048576" sheet="BSCR Source Data"/>
   </cacheSource>
   <cacheFields count="11">
     <cacheField name="cntrycode" numFmtId="0">
@@ -10565,15 +10565,15 @@
         <v>6</v>
       </c>
       <c r="C2" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A2,'Sheet1'!$C:$C,$B2,'Sheet1'!$G:$G,$F2)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A2,'BSCR Source Data'!$C:$C,$B2,'BSCR Source Data'!$G:$G,$F2)</f>
         <v>4645929142.03575</v>
       </c>
       <c r="D2" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A2,'Sheet1'!$C:$C,$B2,'Sheet1'!$G:$G,$F2)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A2,'BSCR Source Data'!$C:$C,$B2,'BSCR Source Data'!$G:$G,$F2)</f>
         <v>2931952651.02002</v>
       </c>
       <c r="E2">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A2,'Sheet1'!$C:$C,$B2,'Sheet1'!$G:$G,$F2)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A2,'BSCR Source Data'!$C:$C,$B2,'BSCR Source Data'!$G:$G,$F2)</f>
         <v>663</v>
       </c>
       <c r="F2">
@@ -10604,15 +10604,15 @@
         <v>6</v>
       </c>
       <c r="C3" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A3,'Sheet1'!$C:$C,$B3,'Sheet1'!$G:$G,$F3)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A3,'BSCR Source Data'!$C:$C,$B3,'BSCR Source Data'!$G:$G,$F3)</f>
         <v>25152755366.6675</v>
       </c>
       <c r="D3" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A3,'Sheet1'!$C:$C,$B3,'Sheet1'!$G:$G,$F3)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A3,'BSCR Source Data'!$C:$C,$B3,'BSCR Source Data'!$G:$G,$F3)</f>
         <v>18626528497.3074</v>
       </c>
       <c r="E3">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A3,'Sheet1'!$C:$C,$B3,'Sheet1'!$G:$G,$F3)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A3,'BSCR Source Data'!$C:$C,$B3,'BSCR Source Data'!$G:$G,$F3)</f>
         <v>4678</v>
       </c>
       <c r="F3">
@@ -10643,15 +10643,15 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A4,'Sheet1'!$C:$C,$B4,'Sheet1'!$G:$G,$F4)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A4,'BSCR Source Data'!$C:$C,$B4,'BSCR Source Data'!$G:$G,$F4)</f>
         <v>1652000</v>
       </c>
       <c r="D4">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A4,'Sheet1'!$C:$C,$B4,'Sheet1'!$G:$G,$F4)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A4,'BSCR Source Data'!$C:$C,$B4,'BSCR Source Data'!$G:$G,$F4)</f>
         <v>1652000</v>
       </c>
       <c r="E4">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A4,'Sheet1'!$C:$C,$B4,'Sheet1'!$G:$G,$F4)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A4,'BSCR Source Data'!$C:$C,$B4,'BSCR Source Data'!$G:$G,$F4)</f>
         <v>9</v>
       </c>
       <c r="F4">
@@ -10682,15 +10682,15 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A5,'Sheet1'!$C:$C,$B5,'Sheet1'!$G:$G,$F5)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A5,'BSCR Source Data'!$C:$C,$B5,'BSCR Source Data'!$G:$G,$F5)</f>
         <v>20414496.8</v>
       </c>
       <c r="D5">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A5,'Sheet1'!$C:$C,$B5,'Sheet1'!$G:$G,$F5)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A5,'BSCR Source Data'!$C:$C,$B5,'BSCR Source Data'!$G:$G,$F5)</f>
         <v>20414496.8</v>
       </c>
       <c r="E5">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A5,'Sheet1'!$C:$C,$B5,'Sheet1'!$G:$G,$F5)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A5,'BSCR Source Data'!$C:$C,$B5,'BSCR Source Data'!$G:$G,$F5)</f>
         <v>27</v>
       </c>
       <c r="F5">
@@ -10721,15 +10721,15 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A6,'Sheet1'!$C:$C,$B6,'Sheet1'!$G:$G,$F6)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A6,'BSCR Source Data'!$C:$C,$B6,'BSCR Source Data'!$G:$G,$F6)</f>
         <v>15433806.4</v>
       </c>
       <c r="D6">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A6,'Sheet1'!$C:$C,$B6,'Sheet1'!$G:$G,$F6)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A6,'BSCR Source Data'!$C:$C,$B6,'BSCR Source Data'!$G:$G,$F6)</f>
         <v>15433806.4</v>
       </c>
       <c r="E6">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A6,'Sheet1'!$C:$C,$B6,'Sheet1'!$G:$G,$F6)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A6,'BSCR Source Data'!$C:$C,$B6,'BSCR Source Data'!$G:$G,$F6)</f>
         <v>29</v>
       </c>
       <c r="F6">
@@ -10760,15 +10760,15 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A7,'Sheet1'!$C:$C,$B7,'Sheet1'!$G:$G,$F7)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A7,'BSCR Source Data'!$C:$C,$B7,'BSCR Source Data'!$G:$G,$F7)</f>
         <v>121728008563.88</v>
       </c>
       <c r="D7">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A7,'Sheet1'!$C:$C,$B7,'Sheet1'!$G:$G,$F7)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A7,'BSCR Source Data'!$C:$C,$B7,'BSCR Source Data'!$G:$G,$F7)</f>
         <v>121728008563.88</v>
       </c>
       <c r="E7">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A7,'Sheet1'!$C:$C,$B7,'Sheet1'!$G:$G,$F7)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A7,'BSCR Source Data'!$C:$C,$B7,'BSCR Source Data'!$G:$G,$F7)</f>
         <v>173658</v>
       </c>
       <c r="F7">
@@ -10799,15 +10799,15 @@
         <v>6</v>
       </c>
       <c r="C8">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A8,'Sheet1'!$C:$C,$B8,'Sheet1'!$G:$G,$F8)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A8,'BSCR Source Data'!$C:$C,$B8,'BSCR Source Data'!$G:$G,$F8)</f>
         <v>699027304.76611</v>
       </c>
       <c r="D8">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A8,'Sheet1'!$C:$C,$B8,'Sheet1'!$G:$G,$F8)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A8,'BSCR Source Data'!$C:$C,$B8,'BSCR Source Data'!$G:$G,$F8)</f>
         <v>406962151.02611</v>
       </c>
       <c r="E8">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A8,'Sheet1'!$C:$C,$B8,'Sheet1'!$G:$G,$F8)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A8,'BSCR Source Data'!$C:$C,$B8,'BSCR Source Data'!$G:$G,$F8)</f>
         <v>55</v>
       </c>
       <c r="F8">
@@ -10838,15 +10838,15 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A9,'Sheet1'!$C:$C,$B9,'Sheet1'!$G:$G,$F9)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A9,'BSCR Source Data'!$C:$C,$B9,'BSCR Source Data'!$G:$G,$F9)</f>
         <v>7347517214.04485</v>
       </c>
       <c r="D9">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A9,'Sheet1'!$C:$C,$B9,'Sheet1'!$G:$G,$F9)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A9,'BSCR Source Data'!$C:$C,$B9,'BSCR Source Data'!$G:$G,$F9)</f>
         <v>5831772777.39485</v>
       </c>
       <c r="E9">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A9,'Sheet1'!$C:$C,$B9,'Sheet1'!$G:$G,$F9)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A9,'BSCR Source Data'!$C:$C,$B9,'BSCR Source Data'!$G:$G,$F9)</f>
         <v>1915</v>
       </c>
       <c r="F9">
@@ -10877,15 +10877,15 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A10,'Sheet1'!$C:$C,$B10,'Sheet1'!$G:$G,$F10)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A10,'BSCR Source Data'!$C:$C,$B10,'BSCR Source Data'!$G:$G,$F10)</f>
         <v>349291128.7</v>
       </c>
       <c r="D10">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A10,'Sheet1'!$C:$C,$B10,'Sheet1'!$G:$G,$F10)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A10,'BSCR Source Data'!$C:$C,$B10,'BSCR Source Data'!$G:$G,$F10)</f>
         <v>349291128.7</v>
       </c>
       <c r="E10">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A10,'Sheet1'!$C:$C,$B10,'Sheet1'!$G:$G,$F10)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A10,'BSCR Source Data'!$C:$C,$B10,'BSCR Source Data'!$G:$G,$F10)</f>
         <v>201</v>
       </c>
       <c r="F10">
@@ -10916,15 +10916,15 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A11,'Sheet1'!$C:$C,$B11,'Sheet1'!$G:$G,$F11)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A11,'BSCR Source Data'!$C:$C,$B11,'BSCR Source Data'!$G:$G,$F11)</f>
         <v>77211907518.142</v>
       </c>
       <c r="D11">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A11,'Sheet1'!$C:$C,$B11,'Sheet1'!$G:$G,$F11)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A11,'BSCR Source Data'!$C:$C,$B11,'BSCR Source Data'!$G:$G,$F11)</f>
         <v>75515308381.742</v>
       </c>
       <c r="E11">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A11,'Sheet1'!$C:$C,$B11,'Sheet1'!$G:$G,$F11)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A11,'BSCR Source Data'!$C:$C,$B11,'BSCR Source Data'!$G:$G,$F11)</f>
         <v>89851</v>
       </c>
       <c r="F11">
@@ -10955,15 +10955,15 @@
         <v>10</v>
       </c>
       <c r="C12" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A12,'Sheet1'!$C:$C,$B12,'Sheet1'!$G:$G,$F12)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A12,'BSCR Source Data'!$C:$C,$B12,'BSCR Source Data'!$G:$G,$F12)</f>
         <v>591803570.7403</v>
       </c>
       <c r="D12" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A12,'Sheet1'!$C:$C,$B12,'Sheet1'!$G:$G,$F12)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A12,'BSCR Source Data'!$C:$C,$B12,'BSCR Source Data'!$G:$G,$F12)</f>
         <v>395404009.102</v>
       </c>
       <c r="E12">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A12,'Sheet1'!$C:$C,$B12,'Sheet1'!$G:$G,$F12)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A12,'BSCR Source Data'!$C:$C,$B12,'BSCR Source Data'!$G:$G,$F12)</f>
         <v>46</v>
       </c>
       <c r="F12">
@@ -10994,15 +10994,15 @@
         <v>10</v>
       </c>
       <c r="C13" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A13,'Sheet1'!$C:$C,$B13,'Sheet1'!$G:$G,$F13)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A13,'BSCR Source Data'!$C:$C,$B13,'BSCR Source Data'!$G:$G,$F13)</f>
         <v>15621176039.34</v>
       </c>
       <c r="D13" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A13,'Sheet1'!$C:$C,$B13,'Sheet1'!$G:$G,$F13)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A13,'BSCR Source Data'!$C:$C,$B13,'BSCR Source Data'!$G:$G,$F13)</f>
         <v>12132651704.25</v>
       </c>
       <c r="E13">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A13,'Sheet1'!$C:$C,$B13,'Sheet1'!$G:$G,$F13)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A13,'BSCR Source Data'!$C:$C,$B13,'BSCR Source Data'!$G:$G,$F13)</f>
         <v>2767</v>
       </c>
       <c r="F13">
@@ -11033,15 +11033,15 @@
         <v>10</v>
       </c>
       <c r="C14">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A14,'Sheet1'!$C:$C,$B14,'Sheet1'!$G:$G,$F14)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A14,'BSCR Source Data'!$C:$C,$B14,'BSCR Source Data'!$G:$G,$F14)</f>
         <v>5578000</v>
       </c>
       <c r="D14">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A14,'Sheet1'!$C:$C,$B14,'Sheet1'!$G:$G,$F14)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A14,'BSCR Source Data'!$C:$C,$B14,'BSCR Source Data'!$G:$G,$F14)</f>
         <v>5578000</v>
       </c>
       <c r="E14">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A14,'Sheet1'!$C:$C,$B14,'Sheet1'!$G:$G,$F14)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A14,'BSCR Source Data'!$C:$C,$B14,'BSCR Source Data'!$G:$G,$F14)</f>
         <v>5</v>
       </c>
       <c r="F14">
@@ -11072,15 +11072,15 @@
         <v>10</v>
       </c>
       <c r="C15">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A15,'Sheet1'!$C:$C,$B15,'Sheet1'!$G:$G,$F15)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A15,'BSCR Source Data'!$C:$C,$B15,'BSCR Source Data'!$G:$G,$F15)</f>
         <v>7099946</v>
       </c>
       <c r="D15">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A15,'Sheet1'!$C:$C,$B15,'Sheet1'!$G:$G,$F15)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A15,'BSCR Source Data'!$C:$C,$B15,'BSCR Source Data'!$G:$G,$F15)</f>
         <v>7099946</v>
       </c>
       <c r="E15">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A15,'Sheet1'!$C:$C,$B15,'Sheet1'!$G:$G,$F15)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A15,'BSCR Source Data'!$C:$C,$B15,'BSCR Source Data'!$G:$G,$F15)</f>
         <v>15</v>
       </c>
       <c r="F15">
@@ -11111,15 +11111,15 @@
         <v>10</v>
       </c>
       <c r="C16">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A16,'Sheet1'!$C:$C,$B16,'Sheet1'!$G:$G,$F16)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A16,'BSCR Source Data'!$C:$C,$B16,'BSCR Source Data'!$G:$G,$F16)</f>
         <v>121288000000</v>
       </c>
       <c r="D16">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A16,'Sheet1'!$C:$C,$B16,'Sheet1'!$G:$G,$F16)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A16,'BSCR Source Data'!$C:$C,$B16,'BSCR Source Data'!$G:$G,$F16)</f>
         <v>121288000000</v>
       </c>
       <c r="E16">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A16,'Sheet1'!$C:$C,$B16,'Sheet1'!$G:$G,$F16)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A16,'BSCR Source Data'!$C:$C,$B16,'BSCR Source Data'!$G:$G,$F16)</f>
         <v>173171</v>
       </c>
       <c r="F16">
@@ -11150,15 +11150,15 @@
         <v>10</v>
       </c>
       <c r="C17">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A17,'Sheet1'!$C:$C,$B17,'Sheet1'!$G:$G,$F17)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A17,'BSCR Source Data'!$C:$C,$B17,'BSCR Source Data'!$G:$G,$F17)</f>
         <v>210175711.428</v>
       </c>
       <c r="D17">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A17,'Sheet1'!$C:$C,$B17,'Sheet1'!$G:$G,$F17)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A17,'BSCR Source Data'!$C:$C,$B17,'BSCR Source Data'!$G:$G,$F17)</f>
         <v>112614669.918</v>
       </c>
       <c r="E17">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A17,'Sheet1'!$C:$C,$B17,'Sheet1'!$G:$G,$F17)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A17,'BSCR Source Data'!$C:$C,$B17,'BSCR Source Data'!$G:$G,$F17)</f>
         <v>11</v>
       </c>
       <c r="F17">
@@ -11189,15 +11189,15 @@
         <v>10</v>
       </c>
       <c r="C18">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A18,'Sheet1'!$C:$C,$B18,'Sheet1'!$G:$G,$F18)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A18,'BSCR Source Data'!$C:$C,$B18,'BSCR Source Data'!$G:$G,$F18)</f>
         <v>2859865269.5161</v>
       </c>
       <c r="D18">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A18,'Sheet1'!$C:$C,$B18,'Sheet1'!$G:$G,$F18)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A18,'BSCR Source Data'!$C:$C,$B18,'BSCR Source Data'!$G:$G,$F18)</f>
         <v>2193629057.0861</v>
       </c>
       <c r="E18">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A18,'Sheet1'!$C:$C,$B18,'Sheet1'!$G:$G,$F18)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A18,'BSCR Source Data'!$C:$C,$B18,'BSCR Source Data'!$G:$G,$F18)</f>
         <v>612</v>
       </c>
       <c r="F18">
@@ -11228,15 +11228,15 @@
         <v>10</v>
       </c>
       <c r="C19">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A19,'Sheet1'!$C:$C,$B19,'Sheet1'!$G:$G,$F19)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A19,'BSCR Source Data'!$C:$C,$B19,'BSCR Source Data'!$G:$G,$F19)</f>
         <v>75479150</v>
       </c>
       <c r="D19">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A19,'Sheet1'!$C:$C,$B19,'Sheet1'!$G:$G,$F19)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A19,'BSCR Source Data'!$C:$C,$B19,'BSCR Source Data'!$G:$G,$F19)</f>
         <v>75479150</v>
       </c>
       <c r="E19">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A19,'Sheet1'!$C:$C,$B19,'Sheet1'!$G:$G,$F19)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A19,'BSCR Source Data'!$C:$C,$B19,'BSCR Source Data'!$G:$G,$F19)</f>
         <v>112</v>
       </c>
       <c r="F19">
@@ -11267,15 +11267,15 @@
         <v>10</v>
       </c>
       <c r="C20">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A20,'Sheet1'!$C:$C,$B20,'Sheet1'!$G:$G,$F20)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A20,'BSCR Source Data'!$C:$C,$B20,'BSCR Source Data'!$G:$G,$F20)</f>
         <v>56019841640.34</v>
       </c>
       <c r="D20">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A20,'Sheet1'!$C:$C,$B20,'Sheet1'!$G:$G,$F20)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A20,'BSCR Source Data'!$C:$C,$B20,'BSCR Source Data'!$G:$G,$F20)</f>
         <v>54739890726.34</v>
       </c>
       <c r="E20">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A20,'Sheet1'!$C:$C,$B20,'Sheet1'!$G:$G,$F20)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A20,'BSCR Source Data'!$C:$C,$B20,'BSCR Source Data'!$G:$G,$F20)</f>
         <v>67520</v>
       </c>
       <c r="F20">
@@ -11306,15 +11306,15 @@
         <v>11</v>
       </c>
       <c r="C21" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A21,'Sheet1'!$C:$C,$B21,'Sheet1'!$G:$G,$F21)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A21,'BSCR Source Data'!$C:$C,$B21,'BSCR Source Data'!$G:$G,$F21)</f>
         <v>3060082.643</v>
       </c>
       <c r="D21" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A21,'Sheet1'!$C:$C,$B21,'Sheet1'!$G:$G,$F21)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A21,'BSCR Source Data'!$C:$C,$B21,'BSCR Source Data'!$G:$G,$F21)</f>
         <v>1599407.467</v>
       </c>
       <c r="E21">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A21,'Sheet1'!$C:$C,$B21,'Sheet1'!$G:$G,$F21)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A21,'BSCR Source Data'!$C:$C,$B21,'BSCR Source Data'!$G:$G,$F21)</f>
         <v>3</v>
       </c>
       <c r="F21">
@@ -11345,15 +11345,15 @@
         <v>11</v>
       </c>
       <c r="C22" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A22,'Sheet1'!$C:$C,$B22,'Sheet1'!$G:$G,$F22)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A22,'BSCR Source Data'!$C:$C,$B22,'BSCR Source Data'!$G:$G,$F22)</f>
         <v>83586974.9</v>
       </c>
       <c r="D22" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A22,'Sheet1'!$C:$C,$B22,'Sheet1'!$G:$G,$F22)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A22,'BSCR Source Data'!$C:$C,$B22,'BSCR Source Data'!$G:$G,$F22)</f>
         <v>47547711</v>
       </c>
       <c r="E22">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A22,'Sheet1'!$C:$C,$B22,'Sheet1'!$G:$G,$F22)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A22,'BSCR Source Data'!$C:$C,$B22,'BSCR Source Data'!$G:$G,$F22)</f>
         <v>10</v>
       </c>
       <c r="F22">
@@ -11384,15 +11384,15 @@
         <v>11</v>
       </c>
       <c r="C23">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A23,'Sheet1'!$C:$C,$B23,'Sheet1'!$G:$G,$F23)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A23,'BSCR Source Data'!$C:$C,$B23,'BSCR Source Data'!$G:$G,$F23)</f>
         <v>276000</v>
       </c>
       <c r="D23">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A23,'Sheet1'!$C:$C,$B23,'Sheet1'!$G:$G,$F23)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A23,'BSCR Source Data'!$C:$C,$B23,'BSCR Source Data'!$G:$G,$F23)</f>
         <v>276000</v>
       </c>
       <c r="E23">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A23,'Sheet1'!$C:$C,$B23,'Sheet1'!$G:$G,$F23)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A23,'BSCR Source Data'!$C:$C,$B23,'BSCR Source Data'!$G:$G,$F23)</f>
         <v>2</v>
       </c>
       <c r="F23">
@@ -11423,15 +11423,15 @@
         <v>11</v>
       </c>
       <c r="C24">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A24,'Sheet1'!$C:$C,$B24,'Sheet1'!$G:$G,$F24)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A24,'BSCR Source Data'!$C:$C,$B24,'BSCR Source Data'!$G:$G,$F24)</f>
         <v>183525417</v>
       </c>
       <c r="D24">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A24,'Sheet1'!$C:$C,$B24,'Sheet1'!$G:$G,$F24)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A24,'BSCR Source Data'!$C:$C,$B24,'BSCR Source Data'!$G:$G,$F24)</f>
         <v>107035050.9</v>
       </c>
       <c r="E24">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A24,'Sheet1'!$C:$C,$B24,'Sheet1'!$G:$G,$F24)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A24,'BSCR Source Data'!$C:$C,$B24,'BSCR Source Data'!$G:$G,$F24)</f>
         <v>42</v>
       </c>
       <c r="F24">
@@ -11462,15 +11462,15 @@
         <v>11</v>
       </c>
       <c r="C25">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A25,'Sheet1'!$C:$C,$B25,'Sheet1'!$G:$G,$F25)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A25,'BSCR Source Data'!$C:$C,$B25,'BSCR Source Data'!$G:$G,$F25)</f>
         <v>20201080.8</v>
       </c>
       <c r="D25">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A25,'Sheet1'!$C:$C,$B25,'Sheet1'!$G:$G,$F25)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A25,'BSCR Source Data'!$C:$C,$B25,'BSCR Source Data'!$G:$G,$F25)</f>
         <v>20201080.8</v>
       </c>
       <c r="E25">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A25,'Sheet1'!$C:$C,$B25,'Sheet1'!$G:$G,$F25)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A25,'BSCR Source Data'!$C:$C,$B25,'BSCR Source Data'!$G:$G,$F25)</f>
         <v>23</v>
       </c>
       <c r="F25">
@@ -11501,15 +11501,15 @@
         <v>12</v>
       </c>
       <c r="C26" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A26,'Sheet1'!$C:$C,$B26,'Sheet1'!$G:$G,$F26)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A26,'BSCR Source Data'!$C:$C,$B26,'BSCR Source Data'!$G:$G,$F26)</f>
         <v>18301343.57</v>
       </c>
       <c r="D26" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A26,'Sheet1'!$C:$C,$B26,'Sheet1'!$G:$G,$F26)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A26,'BSCR Source Data'!$C:$C,$B26,'BSCR Source Data'!$G:$G,$F26)</f>
         <v>16479715.69</v>
       </c>
       <c r="E26">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A26,'Sheet1'!$C:$C,$B26,'Sheet1'!$G:$G,$F26)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A26,'BSCR Source Data'!$C:$C,$B26,'BSCR Source Data'!$G:$G,$F26)</f>
         <v>4</v>
       </c>
       <c r="F26">
@@ -11540,15 +11540,15 @@
         <v>12</v>
       </c>
       <c r="C27" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A27,'Sheet1'!$C:$C,$B27,'Sheet1'!$G:$G,$F27)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A27,'BSCR Source Data'!$C:$C,$B27,'BSCR Source Data'!$G:$G,$F27)</f>
         <v>210957528.1</v>
       </c>
       <c r="D27" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A27,'Sheet1'!$C:$C,$B27,'Sheet1'!$G:$G,$F27)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A27,'BSCR Source Data'!$C:$C,$B27,'BSCR Source Data'!$G:$G,$F27)</f>
         <v>106631319.7</v>
       </c>
       <c r="E27">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A27,'Sheet1'!$C:$C,$B27,'Sheet1'!$G:$G,$F27)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A27,'BSCR Source Data'!$C:$C,$B27,'BSCR Source Data'!$G:$G,$F27)</f>
         <v>18</v>
       </c>
       <c r="F27">
@@ -11579,15 +11579,15 @@
         <v>12</v>
       </c>
       <c r="C28">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A28,'Sheet1'!$C:$C,$B28,'Sheet1'!$G:$G,$F28)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A28,'BSCR Source Data'!$C:$C,$B28,'BSCR Source Data'!$G:$G,$F28)</f>
         <v>110000</v>
       </c>
       <c r="D28">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A28,'Sheet1'!$C:$C,$B28,'Sheet1'!$G:$G,$F28)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A28,'BSCR Source Data'!$C:$C,$B28,'BSCR Source Data'!$G:$G,$F28)</f>
         <v>110000</v>
       </c>
       <c r="E28">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A28,'Sheet1'!$C:$C,$B28,'Sheet1'!$G:$G,$F28)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A28,'BSCR Source Data'!$C:$C,$B28,'BSCR Source Data'!$G:$G,$F28)</f>
         <v>1</v>
       </c>
       <c r="F28">
@@ -11618,15 +11618,15 @@
         <v>12</v>
       </c>
       <c r="C29">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A29,'Sheet1'!$C:$C,$B29,'Sheet1'!$G:$G,$F29)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A29,'BSCR Source Data'!$C:$C,$B29,'BSCR Source Data'!$G:$G,$F29)</f>
         <v>110000</v>
       </c>
       <c r="D29">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A29,'Sheet1'!$C:$C,$B29,'Sheet1'!$G:$G,$F29)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A29,'BSCR Source Data'!$C:$C,$B29,'BSCR Source Data'!$G:$G,$F29)</f>
         <v>110000</v>
       </c>
       <c r="E29">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A29,'Sheet1'!$C:$C,$B29,'Sheet1'!$G:$G,$F29)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A29,'BSCR Source Data'!$C:$C,$B29,'BSCR Source Data'!$G:$G,$F29)</f>
         <v>1</v>
       </c>
       <c r="F29">
@@ -11657,15 +11657,15 @@
         <v>12</v>
       </c>
       <c r="C30">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A30,'Sheet1'!$C:$C,$B30,'Sheet1'!$G:$G,$F30)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A30,'BSCR Source Data'!$C:$C,$B30,'BSCR Source Data'!$G:$G,$F30)</f>
         <v>212000</v>
       </c>
       <c r="D30">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A30,'Sheet1'!$C:$C,$B30,'Sheet1'!$G:$G,$F30)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A30,'BSCR Source Data'!$C:$C,$B30,'BSCR Source Data'!$G:$G,$F30)</f>
         <v>212000</v>
       </c>
       <c r="E30">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A30,'Sheet1'!$C:$C,$B30,'Sheet1'!$G:$G,$F30)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A30,'BSCR Source Data'!$C:$C,$B30,'BSCR Source Data'!$G:$G,$F30)</f>
         <v>1</v>
       </c>
       <c r="F30">
@@ -11696,15 +11696,15 @@
         <v>12</v>
       </c>
       <c r="C31">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A31,'Sheet1'!$C:$C,$B31,'Sheet1'!$G:$G,$F31)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A31,'BSCR Source Data'!$C:$C,$B31,'BSCR Source Data'!$G:$G,$F31)</f>
         <v>7558346.16</v>
       </c>
       <c r="D31">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A31,'Sheet1'!$C:$C,$B31,'Sheet1'!$G:$G,$F31)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A31,'BSCR Source Data'!$C:$C,$B31,'BSCR Source Data'!$G:$G,$F31)</f>
         <v>7558346.16</v>
       </c>
       <c r="E31">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A31,'Sheet1'!$C:$C,$B31,'Sheet1'!$G:$G,$F31)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A31,'BSCR Source Data'!$C:$C,$B31,'BSCR Source Data'!$G:$G,$F31)</f>
         <v>4</v>
       </c>
       <c r="F31">
@@ -11735,15 +11735,15 @@
         <v>12</v>
       </c>
       <c r="C32">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A32,'Sheet1'!$C:$C,$B32,'Sheet1'!$G:$G,$F32)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A32,'BSCR Source Data'!$C:$C,$B32,'BSCR Source Data'!$G:$G,$F32)</f>
         <v>560000</v>
       </c>
       <c r="D32">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A32,'Sheet1'!$C:$C,$B32,'Sheet1'!$G:$G,$F32)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A32,'BSCR Source Data'!$C:$C,$B32,'BSCR Source Data'!$G:$G,$F32)</f>
         <v>560000</v>
       </c>
       <c r="E32">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A32,'Sheet1'!$C:$C,$B32,'Sheet1'!$G:$G,$F32)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A32,'BSCR Source Data'!$C:$C,$B32,'BSCR Source Data'!$G:$G,$F32)</f>
         <v>2</v>
       </c>
       <c r="F32">
@@ -11774,15 +11774,15 @@
         <v>13</v>
       </c>
       <c r="C33" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A33,'Sheet1'!$C:$C,$B33,'Sheet1'!$G:$G,$F33)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A33,'BSCR Source Data'!$C:$C,$B33,'BSCR Source Data'!$G:$G,$F33)</f>
         <v>2372926089.373</v>
       </c>
       <c r="D33" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A33,'Sheet1'!$C:$C,$B33,'Sheet1'!$G:$G,$F33)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A33,'BSCR Source Data'!$C:$C,$B33,'BSCR Source Data'!$G:$G,$F33)</f>
         <v>1420410551.373</v>
       </c>
       <c r="E33">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A33,'Sheet1'!$C:$C,$B33,'Sheet1'!$G:$G,$F33)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A33,'BSCR Source Data'!$C:$C,$B33,'BSCR Source Data'!$G:$G,$F33)</f>
         <v>328</v>
       </c>
       <c r="F33">
@@ -11813,15 +11813,15 @@
         <v>13</v>
       </c>
       <c r="C34" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A34,'Sheet1'!$C:$C,$B34,'Sheet1'!$G:$G,$F34)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A34,'BSCR Source Data'!$C:$C,$B34,'BSCR Source Data'!$G:$G,$F34)</f>
         <v>761662142.89</v>
       </c>
       <c r="D34" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A34,'Sheet1'!$C:$C,$B34,'Sheet1'!$G:$G,$F34)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A34,'BSCR Source Data'!$C:$C,$B34,'BSCR Source Data'!$G:$G,$F34)</f>
         <v>448941035.39</v>
       </c>
       <c r="E34">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A34,'Sheet1'!$C:$C,$B34,'Sheet1'!$G:$G,$F34)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A34,'BSCR Source Data'!$C:$C,$B34,'BSCR Source Data'!$G:$G,$F34)</f>
         <v>119</v>
       </c>
       <c r="F34">
@@ -11852,15 +11852,15 @@
         <v>13</v>
       </c>
       <c r="C35">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A35,'Sheet1'!$C:$C,$B35,'Sheet1'!$G:$G,$F35)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A35,'BSCR Source Data'!$C:$C,$B35,'BSCR Source Data'!$G:$G,$F35)</f>
         <v>545000</v>
       </c>
       <c r="D35">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A35,'Sheet1'!$C:$C,$B35,'Sheet1'!$G:$G,$F35)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A35,'BSCR Source Data'!$C:$C,$B35,'BSCR Source Data'!$G:$G,$F35)</f>
         <v>545000</v>
       </c>
       <c r="E35">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A35,'Sheet1'!$C:$C,$B35,'Sheet1'!$G:$G,$F35)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A35,'BSCR Source Data'!$C:$C,$B35,'BSCR Source Data'!$G:$G,$F35)</f>
         <v>2</v>
       </c>
       <c r="F35">
@@ -11891,15 +11891,15 @@
         <v>13</v>
       </c>
       <c r="C36">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A36,'Sheet1'!$C:$C,$B36,'Sheet1'!$G:$G,$F36)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A36,'BSCR Source Data'!$C:$C,$B36,'BSCR Source Data'!$G:$G,$F36)</f>
         <v>2662700</v>
       </c>
       <c r="D36">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A36,'Sheet1'!$C:$C,$B36,'Sheet1'!$G:$G,$F36)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A36,'BSCR Source Data'!$C:$C,$B36,'BSCR Source Data'!$G:$G,$F36)</f>
         <v>2662700</v>
       </c>
       <c r="E36">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A36,'Sheet1'!$C:$C,$B36,'Sheet1'!$G:$G,$F36)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A36,'BSCR Source Data'!$C:$C,$B36,'BSCR Source Data'!$G:$G,$F36)</f>
         <v>4</v>
       </c>
       <c r="F36">
@@ -11930,15 +11930,15 @@
         <v>13</v>
       </c>
       <c r="C37">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A37,'Sheet1'!$C:$C,$B37,'Sheet1'!$G:$G,$F37)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A37,'BSCR Source Data'!$C:$C,$B37,'BSCR Source Data'!$G:$G,$F37)</f>
         <v>101000</v>
       </c>
       <c r="D37">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A37,'Sheet1'!$C:$C,$B37,'Sheet1'!$G:$G,$F37)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A37,'BSCR Source Data'!$C:$C,$B37,'BSCR Source Data'!$G:$G,$F37)</f>
         <v>101000</v>
       </c>
       <c r="E37">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A37,'Sheet1'!$C:$C,$B37,'Sheet1'!$G:$G,$F37)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A37,'BSCR Source Data'!$C:$C,$B37,'BSCR Source Data'!$G:$G,$F37)</f>
         <v>1</v>
       </c>
       <c r="F37">
@@ -11969,15 +11969,15 @@
         <v>13</v>
       </c>
       <c r="C38">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A38,'Sheet1'!$C:$C,$B38,'Sheet1'!$G:$G,$F38)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A38,'BSCR Source Data'!$C:$C,$B38,'BSCR Source Data'!$G:$G,$F38)</f>
         <v>22746034</v>
       </c>
       <c r="D38">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A38,'Sheet1'!$C:$C,$B38,'Sheet1'!$G:$G,$F38)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A38,'BSCR Source Data'!$C:$C,$B38,'BSCR Source Data'!$G:$G,$F38)</f>
         <v>22746034</v>
       </c>
       <c r="E38">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A38,'Sheet1'!$C:$C,$B38,'Sheet1'!$G:$G,$F38)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A38,'BSCR Source Data'!$C:$C,$B38,'BSCR Source Data'!$G:$G,$F38)</f>
         <v>32</v>
       </c>
       <c r="F38">
@@ -12008,15 +12008,15 @@
         <v>13</v>
       </c>
       <c r="C39">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A39,'Sheet1'!$C:$C,$B39,'Sheet1'!$G:$G,$F39)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A39,'BSCR Source Data'!$C:$C,$B39,'BSCR Source Data'!$G:$G,$F39)</f>
         <v>191741484.23</v>
       </c>
       <c r="D39">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A39,'Sheet1'!$C:$C,$B39,'Sheet1'!$G:$G,$F39)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A39,'BSCR Source Data'!$C:$C,$B39,'BSCR Source Data'!$G:$G,$F39)</f>
         <v>103722849</v>
       </c>
       <c r="E39">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A39,'Sheet1'!$C:$C,$B39,'Sheet1'!$G:$G,$F39)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A39,'BSCR Source Data'!$C:$C,$B39,'BSCR Source Data'!$G:$G,$F39)</f>
         <v>23</v>
       </c>
       <c r="F39">
@@ -12047,15 +12047,15 @@
         <v>13</v>
       </c>
       <c r="C40">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A40,'Sheet1'!$C:$C,$B40,'Sheet1'!$G:$G,$F40)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A40,'BSCR Source Data'!$C:$C,$B40,'BSCR Source Data'!$G:$G,$F40)</f>
         <v>1205659420.15</v>
       </c>
       <c r="D40">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A40,'Sheet1'!$C:$C,$B40,'Sheet1'!$G:$G,$F40)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A40,'BSCR Source Data'!$C:$C,$B40,'BSCR Source Data'!$G:$G,$F40)</f>
         <v>924487181.77</v>
       </c>
       <c r="E40">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A40,'Sheet1'!$C:$C,$B40,'Sheet1'!$G:$G,$F40)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A40,'BSCR Source Data'!$C:$C,$B40,'BSCR Source Data'!$G:$G,$F40)</f>
         <v>318</v>
       </c>
       <c r="F40">
@@ -12086,15 +12086,15 @@
         <v>13</v>
       </c>
       <c r="C41">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A41,'Sheet1'!$C:$C,$B41,'Sheet1'!$G:$G,$F41)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A41,'BSCR Source Data'!$C:$C,$B41,'BSCR Source Data'!$G:$G,$F41)</f>
         <v>107224705.2</v>
       </c>
       <c r="D41">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A41,'Sheet1'!$C:$C,$B41,'Sheet1'!$G:$G,$F41)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A41,'BSCR Source Data'!$C:$C,$B41,'BSCR Source Data'!$G:$G,$F41)</f>
         <v>106417749.2</v>
       </c>
       <c r="E41">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A41,'Sheet1'!$C:$C,$B41,'Sheet1'!$G:$G,$F41)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A41,'BSCR Source Data'!$C:$C,$B41,'BSCR Source Data'!$G:$G,$F41)</f>
         <v>86</v>
       </c>
       <c r="F41">
@@ -12125,15 +12125,15 @@
         <v>14</v>
       </c>
       <c r="C42" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A42,'Sheet1'!$C:$C,$B42,'Sheet1'!$G:$G,$F42)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A42,'BSCR Source Data'!$C:$C,$B42,'BSCR Source Data'!$G:$G,$F42)</f>
         <v>2365811503</v>
       </c>
       <c r="D42" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A42,'Sheet1'!$C:$C,$B42,'Sheet1'!$G:$G,$F42)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A42,'BSCR Source Data'!$C:$C,$B42,'BSCR Source Data'!$G:$G,$F42)</f>
         <v>1413295965</v>
       </c>
       <c r="E42">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A42,'Sheet1'!$C:$C,$B42,'Sheet1'!$G:$G,$F42)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A42,'BSCR Source Data'!$C:$C,$B42,'BSCR Source Data'!$G:$G,$F42)</f>
         <v>326</v>
       </c>
       <c r="F42">
@@ -12164,15 +12164,15 @@
         <v>14</v>
       </c>
       <c r="C43" s="1">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A43,'Sheet1'!$C:$C,$B43,'Sheet1'!$G:$G,$F43)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A43,'BSCR Source Data'!$C:$C,$B43,'BSCR Source Data'!$G:$G,$F43)</f>
         <v>738973417.3</v>
       </c>
       <c r="D43" s="1">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A43,'Sheet1'!$C:$C,$B43,'Sheet1'!$G:$G,$F43)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A43,'BSCR Source Data'!$C:$C,$B43,'BSCR Source Data'!$G:$G,$F43)</f>
         <v>426252309.8</v>
       </c>
       <c r="E43">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A43,'Sheet1'!$C:$C,$B43,'Sheet1'!$G:$G,$F43)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A43,'BSCR Source Data'!$C:$C,$B43,'BSCR Source Data'!$G:$G,$F43)</f>
         <v>106</v>
       </c>
       <c r="F43">
@@ -12203,15 +12203,15 @@
         <v>14</v>
       </c>
       <c r="C44">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A44,'Sheet1'!$C:$C,$B44,'Sheet1'!$G:$G,$F44)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A44,'BSCR Source Data'!$C:$C,$B44,'BSCR Source Data'!$G:$G,$F44)</f>
         <v>345000</v>
       </c>
       <c r="D44">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A44,'Sheet1'!$C:$C,$B44,'Sheet1'!$G:$G,$F44)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A44,'BSCR Source Data'!$C:$C,$B44,'BSCR Source Data'!$G:$G,$F44)</f>
         <v>345000</v>
       </c>
       <c r="E44">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A44,'Sheet1'!$C:$C,$B44,'Sheet1'!$G:$G,$F44)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A44,'BSCR Source Data'!$C:$C,$B44,'BSCR Source Data'!$G:$G,$F44)</f>
         <v>1</v>
       </c>
       <c r="F44">
@@ -12242,15 +12242,15 @@
         <v>14</v>
       </c>
       <c r="C45">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A45,'Sheet1'!$C:$C,$B45,'Sheet1'!$G:$G,$F45)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A45,'BSCR Source Data'!$C:$C,$B45,'BSCR Source Data'!$G:$G,$F45)</f>
         <v>2462700</v>
       </c>
       <c r="D45">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A45,'Sheet1'!$C:$C,$B45,'Sheet1'!$G:$G,$F45)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A45,'BSCR Source Data'!$C:$C,$B45,'BSCR Source Data'!$G:$G,$F45)</f>
         <v>2462700</v>
       </c>
       <c r="E45">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A45,'Sheet1'!$C:$C,$B45,'Sheet1'!$G:$G,$F45)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A45,'BSCR Source Data'!$C:$C,$B45,'BSCR Source Data'!$G:$G,$F45)</f>
         <v>3</v>
       </c>
       <c r="F45">
@@ -12281,15 +12281,15 @@
         <v>14</v>
       </c>
       <c r="C46">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A46,'Sheet1'!$C:$C,$B46,'Sheet1'!$G:$G,$F46)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A46,'BSCR Source Data'!$C:$C,$B46,'BSCR Source Data'!$G:$G,$F46)</f>
         <v>101000</v>
       </c>
       <c r="D46">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A46,'Sheet1'!$C:$C,$B46,'Sheet1'!$G:$G,$F46)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A46,'BSCR Source Data'!$C:$C,$B46,'BSCR Source Data'!$G:$G,$F46)</f>
         <v>101000</v>
       </c>
       <c r="E46">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A46,'Sheet1'!$C:$C,$B46,'Sheet1'!$G:$G,$F46)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A46,'BSCR Source Data'!$C:$C,$B46,'BSCR Source Data'!$G:$G,$F46)</f>
         <v>1</v>
       </c>
       <c r="F46">
@@ -12320,15 +12320,15 @@
         <v>14</v>
       </c>
       <c r="C47">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A47,'Sheet1'!$C:$C,$B47,'Sheet1'!$G:$G,$F47)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A47,'BSCR Source Data'!$C:$C,$B47,'BSCR Source Data'!$G:$G,$F47)</f>
         <v>22746034</v>
       </c>
       <c r="D47">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A47,'Sheet1'!$C:$C,$B47,'Sheet1'!$G:$G,$F47)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A47,'BSCR Source Data'!$C:$C,$B47,'BSCR Source Data'!$G:$G,$F47)</f>
         <v>22746034</v>
       </c>
       <c r="E47">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A47,'Sheet1'!$C:$C,$B47,'Sheet1'!$G:$G,$F47)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A47,'BSCR Source Data'!$C:$C,$B47,'BSCR Source Data'!$G:$G,$F47)</f>
         <v>32</v>
       </c>
       <c r="F47">
@@ -12359,15 +12359,15 @@
         <v>14</v>
       </c>
       <c r="C48">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A48,'Sheet1'!$C:$C,$B48,'Sheet1'!$G:$G,$F48)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A48,'BSCR Source Data'!$C:$C,$B48,'BSCR Source Data'!$G:$G,$F48)</f>
         <v>175292598.8</v>
       </c>
       <c r="D48">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A48,'Sheet1'!$C:$C,$B48,'Sheet1'!$G:$G,$F48)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A48,'BSCR Source Data'!$C:$C,$B48,'BSCR Source Data'!$G:$G,$F48)</f>
         <v>87273963.57</v>
       </c>
       <c r="E48">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A48,'Sheet1'!$C:$C,$B48,'Sheet1'!$G:$G,$F48)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A48,'BSCR Source Data'!$C:$C,$B48,'BSCR Source Data'!$G:$G,$F48)</f>
         <v>20</v>
       </c>
       <c r="F48">
@@ -12398,15 +12398,15 @@
         <v>14</v>
       </c>
       <c r="C49">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A49,'Sheet1'!$C:$C,$B49,'Sheet1'!$G:$G,$F49)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A49,'BSCR Source Data'!$C:$C,$B49,'BSCR Source Data'!$G:$G,$F49)</f>
         <v>906507554.6</v>
       </c>
       <c r="D49">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A49,'Sheet1'!$C:$C,$B49,'Sheet1'!$G:$G,$F49)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A49,'BSCR Source Data'!$C:$C,$B49,'BSCR Source Data'!$G:$G,$F49)</f>
         <v>666539312.4</v>
       </c>
       <c r="E49">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A49,'Sheet1'!$C:$C,$B49,'Sheet1'!$G:$G,$F49)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A49,'BSCR Source Data'!$C:$C,$B49,'BSCR Source Data'!$G:$G,$F49)</f>
         <v>227</v>
       </c>
       <c r="F49">
@@ -12437,15 +12437,15 @@
         <v>14</v>
       </c>
       <c r="C50">
-        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A50,'Sheet1'!$C:$C,$B50,'Sheet1'!$G:$G,$F50)</f>
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A50,'BSCR Source Data'!$C:$C,$B50,'BSCR Source Data'!$G:$G,$F50)</f>
         <v>101774358.8</v>
       </c>
       <c r="D50">
-        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A50,'Sheet1'!$C:$C,$B50,'Sheet1'!$G:$G,$F50)</f>
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A50,'BSCR Source Data'!$C:$C,$B50,'BSCR Source Data'!$G:$G,$F50)</f>
         <v>100967402.8</v>
       </c>
       <c r="E50">
-        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A50,'Sheet1'!$C:$C,$B50,'Sheet1'!$G:$G,$F50)</f>
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A50,'BSCR Source Data'!$C:$C,$B50,'BSCR Source Data'!$G:$G,$F50)</f>
         <v>76</v>
       </c>
       <c r="F50">
@@ -30998,7 +30998,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paste CSV into Sheet1 A:G without replacing formula columns. Formulas apply 1.35 GBP/USD and divide by 1,000,000; output consolidates and piv presents results.</t>
+          <t>Paste the CSV into BSCR Source Data A:G without replacing formula columns. Formulas apply 1.35 GBP/USD and divide by 1,000,000; BSCR Output consolidates and BSCR Pivot Summary presents results.</t>
         </is>
       </c>
     </row>
@@ -31010,7 +31010,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Reviewed piv values are manually entered into the HIC Schedule X workbook. There is no formula link to the final return.</t>
+          <t>Reviewed BSCR Pivot Summary values are manually entered into the HIC Schedule X workbook. There is no formula link to the final return.</t>
         </is>
       </c>
     </row>
@@ -31022,7 +31022,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Refresh output and piv after loading. The checked-in piv is older than Sheet1, so reconcile query, CSV, Sheet1, output, piv and final cells before use.</t>
+          <t>Refresh BSCR Output and BSCR Pivot Summary after loading. The checked-in piv is older than BSCR Source Data, so reconcile query, CSV, BSCR Source Data, BSCR Output, BSCR Pivot Summary and final cells before use.</t>
         </is>
       </c>
     </row>
@@ -31308,11 +31308,11 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -31487,11 +31487,11 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -31558,11 +31558,11 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
         <v>30.8434959</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
         <v>30.8434959</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -31578,11 +31578,11 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
         <v>0.2862</v>
       </c>
       <c r="C5" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
         <v>0.2862</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -31598,11 +31598,11 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
         <v>163747.905595587</v>
       </c>
       <c r="C6" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
         <v>163747.905595587</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -31618,11 +31618,11 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="C7" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -31638,11 +31638,11 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -31757,27 +31757,27 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('output'!$E:$E,'output'!$A:$A,"HIC",'output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>33</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>30.8434959</v>
       </c>
       <c r="D4" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>30.8434959</v>
       </c>
       <c r="E4" s="7">
-        <f>SUMIFS('output'!$E:$E,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")-B4</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-B4</f>
         <v>173654</v>
       </c>
       <c r="F4" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")-C4</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-C4</f>
         <v>164322.324372437</v>
       </c>
       <c r="G4" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")-D4</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-D4</f>
         <v>164322.324372437</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -31817,15 +31817,15 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('output'!$E:$E,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>173687</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="D8" s="7">
-        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="H8" t="inlineStr">

</xml_diff>

<commit_message>
Add BSCR workings instructions tab
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -10,9 +10,10 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30AD028F-592B-4888-AD91-FB2F3163888C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="3" xr2:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="0" xr2:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
   </bookViews>
   <sheets>
+    <sheet name="Instructions" sheetId="10" r:id="rId16"/>
     <sheet name="BSCR Pivot Summary" sheetId="2" r:id="rId1"/>
     <sheet name="BSCR Output" sheetId="1" r:id="rId2"/>
     <sheet name="BSCR Source Data" sheetId="3" r:id="rId3"/>
@@ -10509,6 +10510,183 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="2" max="2" width="115" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>BSCR Workings Instructions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Workbook</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BSCR_Workings.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tab / step</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Purpose and action</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BSCR Source Data</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Paste the BSCR script CSV into A:G only. Expected columns: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Do not overwrite formula columns H:K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BSCR Output</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Formula-driven roll-up by entity, region/peril and geocoding status. Provides gross/net source values plus USD and USD-million values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BSCR Pivot Summary</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Review roll-up of BSCR Output. After loading data, use Data &gt; Refresh All. Treat this as a review view, not the raw source or final return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Refresh after paste</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Use Formulas &gt; Calculate Now or Ctrl+Alt+F9, then Data &gt; Refresh All.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Final template</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Open 2026 BSCR - UKEU - HIC.xlsx. Transfer approved values with Paste Special &gt; Values only; preserve template formatting, formulas and validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Schedule X(a)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>The workings output does not contain approved EP-curve values, annual average loss, standard deviation or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Schedule X(b)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The workings output does not contain the insurance EP curve or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Schedule X(c)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Use the compact Schedule X(c) tab as a regional exposure reference: B4:C4 Atlantic Basin Hurricane; B5:C5 North American Earthquake; B6:C6 European Windstorm; B7:C7 Japanese Earthquake; B8:C8 Japanese Typhoon proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Schedule X(c) limitation</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>The final template separates statutory property premium, all-other premium, statutory property limits and all-other limits. The current output is a combined regional total, so do not paste it into one split row without an approved mapping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Schedule X(f)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Modelability and contract-count classifications are not available from the current BSCR output. Keep those final-template fields pending approved source data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Record the source CSV, run date, row count, gross/net totals, FX basis, operator and reviewer before transferring values.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:B16"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD6788F1-4B47-421A-9EF9-440A877182E4}">
   <sheetPr filterMode="1"/>

</xml_diff>

<commit_message>
Clarify BSCR SQL and workbook input contracts
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -15,8 +15,8 @@
   <sheets>
     <sheet name="Instructions" sheetId="10" r:id="rId16"/>
     <sheet name="BSCR Pivot Summary" sheetId="2" r:id="rId1"/>
-    <sheet name="BSCR Output" sheetId="1" r:id="rId2"/>
-    <sheet name="BSCR Source Data" sheetId="3" r:id="rId3"/>
+    <sheet name="BSCR Output Rollup" sheetId="1" r:id="rId2"/>
+    <sheet name="BSCR Aggregated Input" sheetId="3" r:id="rId3"/>
     <sheet name="AUDIT_SUMMARY" sheetId="4" r:id="rId10"/>
     <sheet name="Settings" sheetId="5" r:id="rId11"/>
     <sheet name="Schedule X(a)" sheetId="6" r:id="rId12"/>
@@ -25,8 +25,8 @@
     <sheet name="Schedule X(f)" sheetId="9" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BSCR Output'!$A$1:$F$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BSCR Source Data'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BSCR Output Rollup'!$A$1:$F$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BSCR Aggregated Input'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
   <pivotCaches>
@@ -1190,7 +1190,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" refreshOnLoad="1" mc:Ignorable="xr" r:id="rId1" refreshedBy="Richard Hampton" refreshedDate="46090.700917708331" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="49" xr:uid="{B1A2DC09-0005-4103-9A04-052000D9B748}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:J50" sheet="BSCR Output"/>
+    <worksheetSource ref="A1:J50" sheet="BSCR Output Rollup"/>
   </cacheSource>
   <cacheFields count="10">
     <cacheField name="bscr_entity" numFmtId="0">
@@ -1298,7 +1298,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" refreshOnLoad="1" mc:Ignorable="xr" r:id="rId1" refreshedBy="Faye Williams" refreshedDate="46106.622011574073" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="453" xr:uid="{8B38D0A1-59CD-453E-BBD5-7D49D4105093}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:K1048576" sheet="BSCR Source Data"/>
+    <worksheetSource ref="A1:K1048576" sheet="BSCR Aggregated Input"/>
   </cacheSource>
   <cacheFields count="11">
     <cacheField name="cntrycode" numFmtId="0">
@@ -10552,138 +10552,162 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BSCR Source Data</t>
+          <t>Raw SQL extract</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paste the BSCR script CSV into A:G only. Expected columns: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Do not overwrite formula columns H:K.</t>
+          <t>bscr-extract.sql produces 8 columns: pml, accgrpid, uwritrname, state, userid1, branchname, cntrycode, is_geocoded. Do not paste this raw SQL CSV directly into the workbook.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BSCR Output</t>
+          <t>Pipeline</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
+        <is>
+          <t>Point BSCR_UKEU.py BSCR_INPUT_CSV at the raw SQL CSV. It classifies, applies retentions and writes output/bscr-output.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BSCR Aggregated Input</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paste generated output/bscr-output.csv into A:G only. Expected headers: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Do not overwrite formula columns H:K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BSCR Output Rollup</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Formula-driven roll-up by entity, region/peril and geocoding status. Provides gross/net source values plus USD and USD-million values.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>BSCR Pivot Summary</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
-          <t>Review roll-up of BSCR Output. After loading data, use Data &gt; Refresh All. Treat this as a review view, not the raw source or final return.</t>
+          <t>Review roll-up of BSCR Output Rollup. After loading data, use Data &gt; Refresh All. Treat this as a review view, not the raw source or final return.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Refresh after paste</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Use Formulas &gt; Calculate Now or Ctrl+Alt+F9, then Data &gt; Refresh All.</t>
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Final template</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Open 2026 BSCR - UKEU - HIC.xlsx. Transfer approved values with Paste Special &gt; Values only; preserve template formatting, formulas and validation.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Schedule X(a)</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>The workings output does not contain approved EP-curve values, annual average loss, standard deviation or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Schedule X(b)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>The workings output does not contain the insurance EP curve or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Schedule X(c)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Use the compact Schedule X(c) tab as a regional exposure reference: B4:C4 Atlantic Basin Hurricane; B5:C5 North American Earthquake; B6:C6 European Windstorm; B7:C7 Japanese Earthquake; B8:C8 Japanese Typhoon proxy.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Schedule X(c) limitation</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>The final template separates statutory property premium, all-other premium, statutory property limits and all-other limits. The current output is a combined regional total, so do not paste it into one split row without an approved mapping.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Schedule X(f)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Modelability and contract-count classifications are not available from the current BSCR output. Keep those final-template fields pending approved source data.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Control</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Record the source CSV, run date, row count, gross/net totals, FX basis, operator and reviewer before transferring values.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B16"/>
+  <autoFilter ref="A4:B18"/>
 </worksheet>
 </file>
 
@@ -10743,15 +10767,15 @@
         <v>6</v>
       </c>
       <c r="C2" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A2,'BSCR Source Data'!$C:$C,$B2,'BSCR Source Data'!$G:$G,$F2)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A2,'BSCR Aggregated Input'!$C:$C,$B2,'BSCR Aggregated Input'!$G:$G,$F2)</f>
         <v>4645929142.03575</v>
       </c>
       <c r="D2" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A2,'BSCR Source Data'!$C:$C,$B2,'BSCR Source Data'!$G:$G,$F2)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A2,'BSCR Aggregated Input'!$C:$C,$B2,'BSCR Aggregated Input'!$G:$G,$F2)</f>
         <v>2931952651.02002</v>
       </c>
       <c r="E2">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A2,'BSCR Source Data'!$C:$C,$B2,'BSCR Source Data'!$G:$G,$F2)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A2,'BSCR Aggregated Input'!$C:$C,$B2,'BSCR Aggregated Input'!$G:$G,$F2)</f>
         <v>663</v>
       </c>
       <c r="F2">
@@ -10782,15 +10806,15 @@
         <v>6</v>
       </c>
       <c r="C3" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A3,'BSCR Source Data'!$C:$C,$B3,'BSCR Source Data'!$G:$G,$F3)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A3,'BSCR Aggregated Input'!$C:$C,$B3,'BSCR Aggregated Input'!$G:$G,$F3)</f>
         <v>25152755366.6675</v>
       </c>
       <c r="D3" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A3,'BSCR Source Data'!$C:$C,$B3,'BSCR Source Data'!$G:$G,$F3)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A3,'BSCR Aggregated Input'!$C:$C,$B3,'BSCR Aggregated Input'!$G:$G,$F3)</f>
         <v>18626528497.3074</v>
       </c>
       <c r="E3">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A3,'BSCR Source Data'!$C:$C,$B3,'BSCR Source Data'!$G:$G,$F3)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A3,'BSCR Aggregated Input'!$C:$C,$B3,'BSCR Aggregated Input'!$G:$G,$F3)</f>
         <v>4678</v>
       </c>
       <c r="F3">
@@ -10821,15 +10845,15 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A4,'BSCR Source Data'!$C:$C,$B4,'BSCR Source Data'!$G:$G,$F4)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A4,'BSCR Aggregated Input'!$C:$C,$B4,'BSCR Aggregated Input'!$G:$G,$F4)</f>
         <v>1652000</v>
       </c>
       <c r="D4">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A4,'BSCR Source Data'!$C:$C,$B4,'BSCR Source Data'!$G:$G,$F4)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A4,'BSCR Aggregated Input'!$C:$C,$B4,'BSCR Aggregated Input'!$G:$G,$F4)</f>
         <v>1652000</v>
       </c>
       <c r="E4">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A4,'BSCR Source Data'!$C:$C,$B4,'BSCR Source Data'!$G:$G,$F4)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A4,'BSCR Aggregated Input'!$C:$C,$B4,'BSCR Aggregated Input'!$G:$G,$F4)</f>
         <v>9</v>
       </c>
       <c r="F4">
@@ -10860,15 +10884,15 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A5,'BSCR Source Data'!$C:$C,$B5,'BSCR Source Data'!$G:$G,$F5)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A5,'BSCR Aggregated Input'!$C:$C,$B5,'BSCR Aggregated Input'!$G:$G,$F5)</f>
         <v>20414496.8</v>
       </c>
       <c r="D5">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A5,'BSCR Source Data'!$C:$C,$B5,'BSCR Source Data'!$G:$G,$F5)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A5,'BSCR Aggregated Input'!$C:$C,$B5,'BSCR Aggregated Input'!$G:$G,$F5)</f>
         <v>20414496.8</v>
       </c>
       <c r="E5">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A5,'BSCR Source Data'!$C:$C,$B5,'BSCR Source Data'!$G:$G,$F5)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A5,'BSCR Aggregated Input'!$C:$C,$B5,'BSCR Aggregated Input'!$G:$G,$F5)</f>
         <v>27</v>
       </c>
       <c r="F5">
@@ -10899,15 +10923,15 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A6,'BSCR Source Data'!$C:$C,$B6,'BSCR Source Data'!$G:$G,$F6)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A6,'BSCR Aggregated Input'!$C:$C,$B6,'BSCR Aggregated Input'!$G:$G,$F6)</f>
         <v>15433806.4</v>
       </c>
       <c r="D6">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A6,'BSCR Source Data'!$C:$C,$B6,'BSCR Source Data'!$G:$G,$F6)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A6,'BSCR Aggregated Input'!$C:$C,$B6,'BSCR Aggregated Input'!$G:$G,$F6)</f>
         <v>15433806.4</v>
       </c>
       <c r="E6">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A6,'BSCR Source Data'!$C:$C,$B6,'BSCR Source Data'!$G:$G,$F6)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A6,'BSCR Aggregated Input'!$C:$C,$B6,'BSCR Aggregated Input'!$G:$G,$F6)</f>
         <v>29</v>
       </c>
       <c r="F6">
@@ -10938,15 +10962,15 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A7,'BSCR Source Data'!$C:$C,$B7,'BSCR Source Data'!$G:$G,$F7)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A7,'BSCR Aggregated Input'!$C:$C,$B7,'BSCR Aggregated Input'!$G:$G,$F7)</f>
         <v>121728008563.88</v>
       </c>
       <c r="D7">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A7,'BSCR Source Data'!$C:$C,$B7,'BSCR Source Data'!$G:$G,$F7)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A7,'BSCR Aggregated Input'!$C:$C,$B7,'BSCR Aggregated Input'!$G:$G,$F7)</f>
         <v>121728008563.88</v>
       </c>
       <c r="E7">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A7,'BSCR Source Data'!$C:$C,$B7,'BSCR Source Data'!$G:$G,$F7)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A7,'BSCR Aggregated Input'!$C:$C,$B7,'BSCR Aggregated Input'!$G:$G,$F7)</f>
         <v>173658</v>
       </c>
       <c r="F7">
@@ -10977,15 +11001,15 @@
         <v>6</v>
       </c>
       <c r="C8">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A8,'BSCR Source Data'!$C:$C,$B8,'BSCR Source Data'!$G:$G,$F8)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A8,'BSCR Aggregated Input'!$C:$C,$B8,'BSCR Aggregated Input'!$G:$G,$F8)</f>
         <v>699027304.76611</v>
       </c>
       <c r="D8">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A8,'BSCR Source Data'!$C:$C,$B8,'BSCR Source Data'!$G:$G,$F8)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A8,'BSCR Aggregated Input'!$C:$C,$B8,'BSCR Aggregated Input'!$G:$G,$F8)</f>
         <v>406962151.02611</v>
       </c>
       <c r="E8">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A8,'BSCR Source Data'!$C:$C,$B8,'BSCR Source Data'!$G:$G,$F8)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A8,'BSCR Aggregated Input'!$C:$C,$B8,'BSCR Aggregated Input'!$G:$G,$F8)</f>
         <v>55</v>
       </c>
       <c r="F8">
@@ -11016,15 +11040,15 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A9,'BSCR Source Data'!$C:$C,$B9,'BSCR Source Data'!$G:$G,$F9)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A9,'BSCR Aggregated Input'!$C:$C,$B9,'BSCR Aggregated Input'!$G:$G,$F9)</f>
         <v>7347517214.04485</v>
       </c>
       <c r="D9">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A9,'BSCR Source Data'!$C:$C,$B9,'BSCR Source Data'!$G:$G,$F9)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A9,'BSCR Aggregated Input'!$C:$C,$B9,'BSCR Aggregated Input'!$G:$G,$F9)</f>
         <v>5831772777.39485</v>
       </c>
       <c r="E9">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A9,'BSCR Source Data'!$C:$C,$B9,'BSCR Source Data'!$G:$G,$F9)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A9,'BSCR Aggregated Input'!$C:$C,$B9,'BSCR Aggregated Input'!$G:$G,$F9)</f>
         <v>1915</v>
       </c>
       <c r="F9">
@@ -11055,15 +11079,15 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A10,'BSCR Source Data'!$C:$C,$B10,'BSCR Source Data'!$G:$G,$F10)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A10,'BSCR Aggregated Input'!$C:$C,$B10,'BSCR Aggregated Input'!$G:$G,$F10)</f>
         <v>349291128.7</v>
       </c>
       <c r="D10">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A10,'BSCR Source Data'!$C:$C,$B10,'BSCR Source Data'!$G:$G,$F10)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A10,'BSCR Aggregated Input'!$C:$C,$B10,'BSCR Aggregated Input'!$G:$G,$F10)</f>
         <v>349291128.7</v>
       </c>
       <c r="E10">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A10,'BSCR Source Data'!$C:$C,$B10,'BSCR Source Data'!$G:$G,$F10)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A10,'BSCR Aggregated Input'!$C:$C,$B10,'BSCR Aggregated Input'!$G:$G,$F10)</f>
         <v>201</v>
       </c>
       <c r="F10">
@@ -11094,15 +11118,15 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A11,'BSCR Source Data'!$C:$C,$B11,'BSCR Source Data'!$G:$G,$F11)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A11,'BSCR Aggregated Input'!$C:$C,$B11,'BSCR Aggregated Input'!$G:$G,$F11)</f>
         <v>77211907518.142</v>
       </c>
       <c r="D11">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A11,'BSCR Source Data'!$C:$C,$B11,'BSCR Source Data'!$G:$G,$F11)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A11,'BSCR Aggregated Input'!$C:$C,$B11,'BSCR Aggregated Input'!$G:$G,$F11)</f>
         <v>75515308381.742</v>
       </c>
       <c r="E11">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A11,'BSCR Source Data'!$C:$C,$B11,'BSCR Source Data'!$G:$G,$F11)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A11,'BSCR Aggregated Input'!$C:$C,$B11,'BSCR Aggregated Input'!$G:$G,$F11)</f>
         <v>89851</v>
       </c>
       <c r="F11">
@@ -11133,15 +11157,15 @@
         <v>10</v>
       </c>
       <c r="C12" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A12,'BSCR Source Data'!$C:$C,$B12,'BSCR Source Data'!$G:$G,$F12)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A12,'BSCR Aggregated Input'!$C:$C,$B12,'BSCR Aggregated Input'!$G:$G,$F12)</f>
         <v>591803570.7403</v>
       </c>
       <c r="D12" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A12,'BSCR Source Data'!$C:$C,$B12,'BSCR Source Data'!$G:$G,$F12)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A12,'BSCR Aggregated Input'!$C:$C,$B12,'BSCR Aggregated Input'!$G:$G,$F12)</f>
         <v>395404009.102</v>
       </c>
       <c r="E12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A12,'BSCR Source Data'!$C:$C,$B12,'BSCR Source Data'!$G:$G,$F12)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A12,'BSCR Aggregated Input'!$C:$C,$B12,'BSCR Aggregated Input'!$G:$G,$F12)</f>
         <v>46</v>
       </c>
       <c r="F12">
@@ -11172,15 +11196,15 @@
         <v>10</v>
       </c>
       <c r="C13" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A13,'BSCR Source Data'!$C:$C,$B13,'BSCR Source Data'!$G:$G,$F13)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A13,'BSCR Aggregated Input'!$C:$C,$B13,'BSCR Aggregated Input'!$G:$G,$F13)</f>
         <v>15621176039.34</v>
       </c>
       <c r="D13" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A13,'BSCR Source Data'!$C:$C,$B13,'BSCR Source Data'!$G:$G,$F13)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A13,'BSCR Aggregated Input'!$C:$C,$B13,'BSCR Aggregated Input'!$G:$G,$F13)</f>
         <v>12132651704.25</v>
       </c>
       <c r="E13">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A13,'BSCR Source Data'!$C:$C,$B13,'BSCR Source Data'!$G:$G,$F13)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A13,'BSCR Aggregated Input'!$C:$C,$B13,'BSCR Aggregated Input'!$G:$G,$F13)</f>
         <v>2767</v>
       </c>
       <c r="F13">
@@ -11211,15 +11235,15 @@
         <v>10</v>
       </c>
       <c r="C14">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A14,'BSCR Source Data'!$C:$C,$B14,'BSCR Source Data'!$G:$G,$F14)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A14,'BSCR Aggregated Input'!$C:$C,$B14,'BSCR Aggregated Input'!$G:$G,$F14)</f>
         <v>5578000</v>
       </c>
       <c r="D14">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A14,'BSCR Source Data'!$C:$C,$B14,'BSCR Source Data'!$G:$G,$F14)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A14,'BSCR Aggregated Input'!$C:$C,$B14,'BSCR Aggregated Input'!$G:$G,$F14)</f>
         <v>5578000</v>
       </c>
       <c r="E14">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A14,'BSCR Source Data'!$C:$C,$B14,'BSCR Source Data'!$G:$G,$F14)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A14,'BSCR Aggregated Input'!$C:$C,$B14,'BSCR Aggregated Input'!$G:$G,$F14)</f>
         <v>5</v>
       </c>
       <c r="F14">
@@ -11250,15 +11274,15 @@
         <v>10</v>
       </c>
       <c r="C15">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A15,'BSCR Source Data'!$C:$C,$B15,'BSCR Source Data'!$G:$G,$F15)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A15,'BSCR Aggregated Input'!$C:$C,$B15,'BSCR Aggregated Input'!$G:$G,$F15)</f>
         <v>7099946</v>
       </c>
       <c r="D15">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A15,'BSCR Source Data'!$C:$C,$B15,'BSCR Source Data'!$G:$G,$F15)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A15,'BSCR Aggregated Input'!$C:$C,$B15,'BSCR Aggregated Input'!$G:$G,$F15)</f>
         <v>7099946</v>
       </c>
       <c r="E15">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A15,'BSCR Source Data'!$C:$C,$B15,'BSCR Source Data'!$G:$G,$F15)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A15,'BSCR Aggregated Input'!$C:$C,$B15,'BSCR Aggregated Input'!$G:$G,$F15)</f>
         <v>15</v>
       </c>
       <c r="F15">
@@ -11289,15 +11313,15 @@
         <v>10</v>
       </c>
       <c r="C16">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A16,'BSCR Source Data'!$C:$C,$B16,'BSCR Source Data'!$G:$G,$F16)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A16,'BSCR Aggregated Input'!$C:$C,$B16,'BSCR Aggregated Input'!$G:$G,$F16)</f>
         <v>121288000000</v>
       </c>
       <c r="D16">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A16,'BSCR Source Data'!$C:$C,$B16,'BSCR Source Data'!$G:$G,$F16)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A16,'BSCR Aggregated Input'!$C:$C,$B16,'BSCR Aggregated Input'!$G:$G,$F16)</f>
         <v>121288000000</v>
       </c>
       <c r="E16">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A16,'BSCR Source Data'!$C:$C,$B16,'BSCR Source Data'!$G:$G,$F16)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A16,'BSCR Aggregated Input'!$C:$C,$B16,'BSCR Aggregated Input'!$G:$G,$F16)</f>
         <v>173171</v>
       </c>
       <c r="F16">
@@ -11328,15 +11352,15 @@
         <v>10</v>
       </c>
       <c r="C17">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A17,'BSCR Source Data'!$C:$C,$B17,'BSCR Source Data'!$G:$G,$F17)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A17,'BSCR Aggregated Input'!$C:$C,$B17,'BSCR Aggregated Input'!$G:$G,$F17)</f>
         <v>210175711.428</v>
       </c>
       <c r="D17">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A17,'BSCR Source Data'!$C:$C,$B17,'BSCR Source Data'!$G:$G,$F17)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A17,'BSCR Aggregated Input'!$C:$C,$B17,'BSCR Aggregated Input'!$G:$G,$F17)</f>
         <v>112614669.918</v>
       </c>
       <c r="E17">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A17,'BSCR Source Data'!$C:$C,$B17,'BSCR Source Data'!$G:$G,$F17)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A17,'BSCR Aggregated Input'!$C:$C,$B17,'BSCR Aggregated Input'!$G:$G,$F17)</f>
         <v>11</v>
       </c>
       <c r="F17">
@@ -11367,15 +11391,15 @@
         <v>10</v>
       </c>
       <c r="C18">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A18,'BSCR Source Data'!$C:$C,$B18,'BSCR Source Data'!$G:$G,$F18)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A18,'BSCR Aggregated Input'!$C:$C,$B18,'BSCR Aggregated Input'!$G:$G,$F18)</f>
         <v>2859865269.5161</v>
       </c>
       <c r="D18">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A18,'BSCR Source Data'!$C:$C,$B18,'BSCR Source Data'!$G:$G,$F18)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A18,'BSCR Aggregated Input'!$C:$C,$B18,'BSCR Aggregated Input'!$G:$G,$F18)</f>
         <v>2193629057.0861</v>
       </c>
       <c r="E18">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A18,'BSCR Source Data'!$C:$C,$B18,'BSCR Source Data'!$G:$G,$F18)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A18,'BSCR Aggregated Input'!$C:$C,$B18,'BSCR Aggregated Input'!$G:$G,$F18)</f>
         <v>612</v>
       </c>
       <c r="F18">
@@ -11406,15 +11430,15 @@
         <v>10</v>
       </c>
       <c r="C19">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A19,'BSCR Source Data'!$C:$C,$B19,'BSCR Source Data'!$G:$G,$F19)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A19,'BSCR Aggregated Input'!$C:$C,$B19,'BSCR Aggregated Input'!$G:$G,$F19)</f>
         <v>75479150</v>
       </c>
       <c r="D19">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A19,'BSCR Source Data'!$C:$C,$B19,'BSCR Source Data'!$G:$G,$F19)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A19,'BSCR Aggregated Input'!$C:$C,$B19,'BSCR Aggregated Input'!$G:$G,$F19)</f>
         <v>75479150</v>
       </c>
       <c r="E19">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A19,'BSCR Source Data'!$C:$C,$B19,'BSCR Source Data'!$G:$G,$F19)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A19,'BSCR Aggregated Input'!$C:$C,$B19,'BSCR Aggregated Input'!$G:$G,$F19)</f>
         <v>112</v>
       </c>
       <c r="F19">
@@ -11445,15 +11469,15 @@
         <v>10</v>
       </c>
       <c r="C20">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A20,'BSCR Source Data'!$C:$C,$B20,'BSCR Source Data'!$G:$G,$F20)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A20,'BSCR Aggregated Input'!$C:$C,$B20,'BSCR Aggregated Input'!$G:$G,$F20)</f>
         <v>56019841640.34</v>
       </c>
       <c r="D20">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A20,'BSCR Source Data'!$C:$C,$B20,'BSCR Source Data'!$G:$G,$F20)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A20,'BSCR Aggregated Input'!$C:$C,$B20,'BSCR Aggregated Input'!$G:$G,$F20)</f>
         <v>54739890726.34</v>
       </c>
       <c r="E20">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A20,'BSCR Source Data'!$C:$C,$B20,'BSCR Source Data'!$G:$G,$F20)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A20,'BSCR Aggregated Input'!$C:$C,$B20,'BSCR Aggregated Input'!$G:$G,$F20)</f>
         <v>67520</v>
       </c>
       <c r="F20">
@@ -11484,15 +11508,15 @@
         <v>11</v>
       </c>
       <c r="C21" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A21,'BSCR Source Data'!$C:$C,$B21,'BSCR Source Data'!$G:$G,$F21)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A21,'BSCR Aggregated Input'!$C:$C,$B21,'BSCR Aggregated Input'!$G:$G,$F21)</f>
         <v>3060082.643</v>
       </c>
       <c r="D21" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A21,'BSCR Source Data'!$C:$C,$B21,'BSCR Source Data'!$G:$G,$F21)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A21,'BSCR Aggregated Input'!$C:$C,$B21,'BSCR Aggregated Input'!$G:$G,$F21)</f>
         <v>1599407.467</v>
       </c>
       <c r="E21">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A21,'BSCR Source Data'!$C:$C,$B21,'BSCR Source Data'!$G:$G,$F21)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A21,'BSCR Aggregated Input'!$C:$C,$B21,'BSCR Aggregated Input'!$G:$G,$F21)</f>
         <v>3</v>
       </c>
       <c r="F21">
@@ -11523,15 +11547,15 @@
         <v>11</v>
       </c>
       <c r="C22" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A22,'BSCR Source Data'!$C:$C,$B22,'BSCR Source Data'!$G:$G,$F22)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A22,'BSCR Aggregated Input'!$C:$C,$B22,'BSCR Aggregated Input'!$G:$G,$F22)</f>
         <v>83586974.9</v>
       </c>
       <c r="D22" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A22,'BSCR Source Data'!$C:$C,$B22,'BSCR Source Data'!$G:$G,$F22)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A22,'BSCR Aggregated Input'!$C:$C,$B22,'BSCR Aggregated Input'!$G:$G,$F22)</f>
         <v>47547711</v>
       </c>
       <c r="E22">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A22,'BSCR Source Data'!$C:$C,$B22,'BSCR Source Data'!$G:$G,$F22)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A22,'BSCR Aggregated Input'!$C:$C,$B22,'BSCR Aggregated Input'!$G:$G,$F22)</f>
         <v>10</v>
       </c>
       <c r="F22">
@@ -11562,15 +11586,15 @@
         <v>11</v>
       </c>
       <c r="C23">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A23,'BSCR Source Data'!$C:$C,$B23,'BSCR Source Data'!$G:$G,$F23)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A23,'BSCR Aggregated Input'!$C:$C,$B23,'BSCR Aggregated Input'!$G:$G,$F23)</f>
         <v>276000</v>
       </c>
       <c r="D23">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A23,'BSCR Source Data'!$C:$C,$B23,'BSCR Source Data'!$G:$G,$F23)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A23,'BSCR Aggregated Input'!$C:$C,$B23,'BSCR Aggregated Input'!$G:$G,$F23)</f>
         <v>276000</v>
       </c>
       <c r="E23">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A23,'BSCR Source Data'!$C:$C,$B23,'BSCR Source Data'!$G:$G,$F23)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A23,'BSCR Aggregated Input'!$C:$C,$B23,'BSCR Aggregated Input'!$G:$G,$F23)</f>
         <v>2</v>
       </c>
       <c r="F23">
@@ -11601,15 +11625,15 @@
         <v>11</v>
       </c>
       <c r="C24">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A24,'BSCR Source Data'!$C:$C,$B24,'BSCR Source Data'!$G:$G,$F24)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A24,'BSCR Aggregated Input'!$C:$C,$B24,'BSCR Aggregated Input'!$G:$G,$F24)</f>
         <v>183525417</v>
       </c>
       <c r="D24">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A24,'BSCR Source Data'!$C:$C,$B24,'BSCR Source Data'!$G:$G,$F24)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A24,'BSCR Aggregated Input'!$C:$C,$B24,'BSCR Aggregated Input'!$G:$G,$F24)</f>
         <v>107035050.9</v>
       </c>
       <c r="E24">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A24,'BSCR Source Data'!$C:$C,$B24,'BSCR Source Data'!$G:$G,$F24)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A24,'BSCR Aggregated Input'!$C:$C,$B24,'BSCR Aggregated Input'!$G:$G,$F24)</f>
         <v>42</v>
       </c>
       <c r="F24">
@@ -11640,15 +11664,15 @@
         <v>11</v>
       </c>
       <c r="C25">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A25,'BSCR Source Data'!$C:$C,$B25,'BSCR Source Data'!$G:$G,$F25)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A25,'BSCR Aggregated Input'!$C:$C,$B25,'BSCR Aggregated Input'!$G:$G,$F25)</f>
         <v>20201080.8</v>
       </c>
       <c r="D25">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A25,'BSCR Source Data'!$C:$C,$B25,'BSCR Source Data'!$G:$G,$F25)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A25,'BSCR Aggregated Input'!$C:$C,$B25,'BSCR Aggregated Input'!$G:$G,$F25)</f>
         <v>20201080.8</v>
       </c>
       <c r="E25">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A25,'BSCR Source Data'!$C:$C,$B25,'BSCR Source Data'!$G:$G,$F25)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A25,'BSCR Aggregated Input'!$C:$C,$B25,'BSCR Aggregated Input'!$G:$G,$F25)</f>
         <v>23</v>
       </c>
       <c r="F25">
@@ -11679,15 +11703,15 @@
         <v>12</v>
       </c>
       <c r="C26" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A26,'BSCR Source Data'!$C:$C,$B26,'BSCR Source Data'!$G:$G,$F26)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A26,'BSCR Aggregated Input'!$C:$C,$B26,'BSCR Aggregated Input'!$G:$G,$F26)</f>
         <v>18301343.57</v>
       </c>
       <c r="D26" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A26,'BSCR Source Data'!$C:$C,$B26,'BSCR Source Data'!$G:$G,$F26)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A26,'BSCR Aggregated Input'!$C:$C,$B26,'BSCR Aggregated Input'!$G:$G,$F26)</f>
         <v>16479715.69</v>
       </c>
       <c r="E26">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A26,'BSCR Source Data'!$C:$C,$B26,'BSCR Source Data'!$G:$G,$F26)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A26,'BSCR Aggregated Input'!$C:$C,$B26,'BSCR Aggregated Input'!$G:$G,$F26)</f>
         <v>4</v>
       </c>
       <c r="F26">
@@ -11718,15 +11742,15 @@
         <v>12</v>
       </c>
       <c r="C27" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A27,'BSCR Source Data'!$C:$C,$B27,'BSCR Source Data'!$G:$G,$F27)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A27,'BSCR Aggregated Input'!$C:$C,$B27,'BSCR Aggregated Input'!$G:$G,$F27)</f>
         <v>210957528.1</v>
       </c>
       <c r="D27" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A27,'BSCR Source Data'!$C:$C,$B27,'BSCR Source Data'!$G:$G,$F27)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A27,'BSCR Aggregated Input'!$C:$C,$B27,'BSCR Aggregated Input'!$G:$G,$F27)</f>
         <v>106631319.7</v>
       </c>
       <c r="E27">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A27,'BSCR Source Data'!$C:$C,$B27,'BSCR Source Data'!$G:$G,$F27)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A27,'BSCR Aggregated Input'!$C:$C,$B27,'BSCR Aggregated Input'!$G:$G,$F27)</f>
         <v>18</v>
       </c>
       <c r="F27">
@@ -11757,15 +11781,15 @@
         <v>12</v>
       </c>
       <c r="C28">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A28,'BSCR Source Data'!$C:$C,$B28,'BSCR Source Data'!$G:$G,$F28)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A28,'BSCR Aggregated Input'!$C:$C,$B28,'BSCR Aggregated Input'!$G:$G,$F28)</f>
         <v>110000</v>
       </c>
       <c r="D28">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A28,'BSCR Source Data'!$C:$C,$B28,'BSCR Source Data'!$G:$G,$F28)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A28,'BSCR Aggregated Input'!$C:$C,$B28,'BSCR Aggregated Input'!$G:$G,$F28)</f>
         <v>110000</v>
       </c>
       <c r="E28">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A28,'BSCR Source Data'!$C:$C,$B28,'BSCR Source Data'!$G:$G,$F28)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A28,'BSCR Aggregated Input'!$C:$C,$B28,'BSCR Aggregated Input'!$G:$G,$F28)</f>
         <v>1</v>
       </c>
       <c r="F28">
@@ -11796,15 +11820,15 @@
         <v>12</v>
       </c>
       <c r="C29">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A29,'BSCR Source Data'!$C:$C,$B29,'BSCR Source Data'!$G:$G,$F29)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A29,'BSCR Aggregated Input'!$C:$C,$B29,'BSCR Aggregated Input'!$G:$G,$F29)</f>
         <v>110000</v>
       </c>
       <c r="D29">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A29,'BSCR Source Data'!$C:$C,$B29,'BSCR Source Data'!$G:$G,$F29)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A29,'BSCR Aggregated Input'!$C:$C,$B29,'BSCR Aggregated Input'!$G:$G,$F29)</f>
         <v>110000</v>
       </c>
       <c r="E29">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A29,'BSCR Source Data'!$C:$C,$B29,'BSCR Source Data'!$G:$G,$F29)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A29,'BSCR Aggregated Input'!$C:$C,$B29,'BSCR Aggregated Input'!$G:$G,$F29)</f>
         <v>1</v>
       </c>
       <c r="F29">
@@ -11835,15 +11859,15 @@
         <v>12</v>
       </c>
       <c r="C30">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A30,'BSCR Source Data'!$C:$C,$B30,'BSCR Source Data'!$G:$G,$F30)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A30,'BSCR Aggregated Input'!$C:$C,$B30,'BSCR Aggregated Input'!$G:$G,$F30)</f>
         <v>212000</v>
       </c>
       <c r="D30">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A30,'BSCR Source Data'!$C:$C,$B30,'BSCR Source Data'!$G:$G,$F30)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A30,'BSCR Aggregated Input'!$C:$C,$B30,'BSCR Aggregated Input'!$G:$G,$F30)</f>
         <v>212000</v>
       </c>
       <c r="E30">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A30,'BSCR Source Data'!$C:$C,$B30,'BSCR Source Data'!$G:$G,$F30)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A30,'BSCR Aggregated Input'!$C:$C,$B30,'BSCR Aggregated Input'!$G:$G,$F30)</f>
         <v>1</v>
       </c>
       <c r="F30">
@@ -11874,15 +11898,15 @@
         <v>12</v>
       </c>
       <c r="C31">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A31,'BSCR Source Data'!$C:$C,$B31,'BSCR Source Data'!$G:$G,$F31)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A31,'BSCR Aggregated Input'!$C:$C,$B31,'BSCR Aggregated Input'!$G:$G,$F31)</f>
         <v>7558346.16</v>
       </c>
       <c r="D31">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A31,'BSCR Source Data'!$C:$C,$B31,'BSCR Source Data'!$G:$G,$F31)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A31,'BSCR Aggregated Input'!$C:$C,$B31,'BSCR Aggregated Input'!$G:$G,$F31)</f>
         <v>7558346.16</v>
       </c>
       <c r="E31">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A31,'BSCR Source Data'!$C:$C,$B31,'BSCR Source Data'!$G:$G,$F31)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A31,'BSCR Aggregated Input'!$C:$C,$B31,'BSCR Aggregated Input'!$G:$G,$F31)</f>
         <v>4</v>
       </c>
       <c r="F31">
@@ -11913,15 +11937,15 @@
         <v>12</v>
       </c>
       <c r="C32">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A32,'BSCR Source Data'!$C:$C,$B32,'BSCR Source Data'!$G:$G,$F32)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A32,'BSCR Aggregated Input'!$C:$C,$B32,'BSCR Aggregated Input'!$G:$G,$F32)</f>
         <v>560000</v>
       </c>
       <c r="D32">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A32,'BSCR Source Data'!$C:$C,$B32,'BSCR Source Data'!$G:$G,$F32)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A32,'BSCR Aggregated Input'!$C:$C,$B32,'BSCR Aggregated Input'!$G:$G,$F32)</f>
         <v>560000</v>
       </c>
       <c r="E32">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A32,'BSCR Source Data'!$C:$C,$B32,'BSCR Source Data'!$G:$G,$F32)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A32,'BSCR Aggregated Input'!$C:$C,$B32,'BSCR Aggregated Input'!$G:$G,$F32)</f>
         <v>2</v>
       </c>
       <c r="F32">
@@ -11952,15 +11976,15 @@
         <v>13</v>
       </c>
       <c r="C33" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A33,'BSCR Source Data'!$C:$C,$B33,'BSCR Source Data'!$G:$G,$F33)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A33,'BSCR Aggregated Input'!$C:$C,$B33,'BSCR Aggregated Input'!$G:$G,$F33)</f>
         <v>2372926089.373</v>
       </c>
       <c r="D33" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A33,'BSCR Source Data'!$C:$C,$B33,'BSCR Source Data'!$G:$G,$F33)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A33,'BSCR Aggregated Input'!$C:$C,$B33,'BSCR Aggregated Input'!$G:$G,$F33)</f>
         <v>1420410551.373</v>
       </c>
       <c r="E33">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A33,'BSCR Source Data'!$C:$C,$B33,'BSCR Source Data'!$G:$G,$F33)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A33,'BSCR Aggregated Input'!$C:$C,$B33,'BSCR Aggregated Input'!$G:$G,$F33)</f>
         <v>328</v>
       </c>
       <c r="F33">
@@ -11991,15 +12015,15 @@
         <v>13</v>
       </c>
       <c r="C34" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A34,'BSCR Source Data'!$C:$C,$B34,'BSCR Source Data'!$G:$G,$F34)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A34,'BSCR Aggregated Input'!$C:$C,$B34,'BSCR Aggregated Input'!$G:$G,$F34)</f>
         <v>761662142.89</v>
       </c>
       <c r="D34" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A34,'BSCR Source Data'!$C:$C,$B34,'BSCR Source Data'!$G:$G,$F34)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A34,'BSCR Aggregated Input'!$C:$C,$B34,'BSCR Aggregated Input'!$G:$G,$F34)</f>
         <v>448941035.39</v>
       </c>
       <c r="E34">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A34,'BSCR Source Data'!$C:$C,$B34,'BSCR Source Data'!$G:$G,$F34)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A34,'BSCR Aggregated Input'!$C:$C,$B34,'BSCR Aggregated Input'!$G:$G,$F34)</f>
         <v>119</v>
       </c>
       <c r="F34">
@@ -12030,15 +12054,15 @@
         <v>13</v>
       </c>
       <c r="C35">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A35,'BSCR Source Data'!$C:$C,$B35,'BSCR Source Data'!$G:$G,$F35)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A35,'BSCR Aggregated Input'!$C:$C,$B35,'BSCR Aggregated Input'!$G:$G,$F35)</f>
         <v>545000</v>
       </c>
       <c r="D35">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A35,'BSCR Source Data'!$C:$C,$B35,'BSCR Source Data'!$G:$G,$F35)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A35,'BSCR Aggregated Input'!$C:$C,$B35,'BSCR Aggregated Input'!$G:$G,$F35)</f>
         <v>545000</v>
       </c>
       <c r="E35">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A35,'BSCR Source Data'!$C:$C,$B35,'BSCR Source Data'!$G:$G,$F35)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A35,'BSCR Aggregated Input'!$C:$C,$B35,'BSCR Aggregated Input'!$G:$G,$F35)</f>
         <v>2</v>
       </c>
       <c r="F35">
@@ -12069,15 +12093,15 @@
         <v>13</v>
       </c>
       <c r="C36">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A36,'BSCR Source Data'!$C:$C,$B36,'BSCR Source Data'!$G:$G,$F36)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A36,'BSCR Aggregated Input'!$C:$C,$B36,'BSCR Aggregated Input'!$G:$G,$F36)</f>
         <v>2662700</v>
       </c>
       <c r="D36">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A36,'BSCR Source Data'!$C:$C,$B36,'BSCR Source Data'!$G:$G,$F36)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A36,'BSCR Aggregated Input'!$C:$C,$B36,'BSCR Aggregated Input'!$G:$G,$F36)</f>
         <v>2662700</v>
       </c>
       <c r="E36">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A36,'BSCR Source Data'!$C:$C,$B36,'BSCR Source Data'!$G:$G,$F36)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A36,'BSCR Aggregated Input'!$C:$C,$B36,'BSCR Aggregated Input'!$G:$G,$F36)</f>
         <v>4</v>
       </c>
       <c r="F36">
@@ -12108,15 +12132,15 @@
         <v>13</v>
       </c>
       <c r="C37">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A37,'BSCR Source Data'!$C:$C,$B37,'BSCR Source Data'!$G:$G,$F37)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A37,'BSCR Aggregated Input'!$C:$C,$B37,'BSCR Aggregated Input'!$G:$G,$F37)</f>
         <v>101000</v>
       </c>
       <c r="D37">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A37,'BSCR Source Data'!$C:$C,$B37,'BSCR Source Data'!$G:$G,$F37)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A37,'BSCR Aggregated Input'!$C:$C,$B37,'BSCR Aggregated Input'!$G:$G,$F37)</f>
         <v>101000</v>
       </c>
       <c r="E37">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A37,'BSCR Source Data'!$C:$C,$B37,'BSCR Source Data'!$G:$G,$F37)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A37,'BSCR Aggregated Input'!$C:$C,$B37,'BSCR Aggregated Input'!$G:$G,$F37)</f>
         <v>1</v>
       </c>
       <c r="F37">
@@ -12147,15 +12171,15 @@
         <v>13</v>
       </c>
       <c r="C38">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A38,'BSCR Source Data'!$C:$C,$B38,'BSCR Source Data'!$G:$G,$F38)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A38,'BSCR Aggregated Input'!$C:$C,$B38,'BSCR Aggregated Input'!$G:$G,$F38)</f>
         <v>22746034</v>
       </c>
       <c r="D38">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A38,'BSCR Source Data'!$C:$C,$B38,'BSCR Source Data'!$G:$G,$F38)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A38,'BSCR Aggregated Input'!$C:$C,$B38,'BSCR Aggregated Input'!$G:$G,$F38)</f>
         <v>22746034</v>
       </c>
       <c r="E38">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A38,'BSCR Source Data'!$C:$C,$B38,'BSCR Source Data'!$G:$G,$F38)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A38,'BSCR Aggregated Input'!$C:$C,$B38,'BSCR Aggregated Input'!$G:$G,$F38)</f>
         <v>32</v>
       </c>
       <c r="F38">
@@ -12186,15 +12210,15 @@
         <v>13</v>
       </c>
       <c r="C39">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A39,'BSCR Source Data'!$C:$C,$B39,'BSCR Source Data'!$G:$G,$F39)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A39,'BSCR Aggregated Input'!$C:$C,$B39,'BSCR Aggregated Input'!$G:$G,$F39)</f>
         <v>191741484.23</v>
       </c>
       <c r="D39">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A39,'BSCR Source Data'!$C:$C,$B39,'BSCR Source Data'!$G:$G,$F39)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A39,'BSCR Aggregated Input'!$C:$C,$B39,'BSCR Aggregated Input'!$G:$G,$F39)</f>
         <v>103722849</v>
       </c>
       <c r="E39">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A39,'BSCR Source Data'!$C:$C,$B39,'BSCR Source Data'!$G:$G,$F39)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A39,'BSCR Aggregated Input'!$C:$C,$B39,'BSCR Aggregated Input'!$G:$G,$F39)</f>
         <v>23</v>
       </c>
       <c r="F39">
@@ -12225,15 +12249,15 @@
         <v>13</v>
       </c>
       <c r="C40">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A40,'BSCR Source Data'!$C:$C,$B40,'BSCR Source Data'!$G:$G,$F40)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A40,'BSCR Aggregated Input'!$C:$C,$B40,'BSCR Aggregated Input'!$G:$G,$F40)</f>
         <v>1205659420.15</v>
       </c>
       <c r="D40">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A40,'BSCR Source Data'!$C:$C,$B40,'BSCR Source Data'!$G:$G,$F40)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A40,'BSCR Aggregated Input'!$C:$C,$B40,'BSCR Aggregated Input'!$G:$G,$F40)</f>
         <v>924487181.77</v>
       </c>
       <c r="E40">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A40,'BSCR Source Data'!$C:$C,$B40,'BSCR Source Data'!$G:$G,$F40)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A40,'BSCR Aggregated Input'!$C:$C,$B40,'BSCR Aggregated Input'!$G:$G,$F40)</f>
         <v>318</v>
       </c>
       <c r="F40">
@@ -12264,15 +12288,15 @@
         <v>13</v>
       </c>
       <c r="C41">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A41,'BSCR Source Data'!$C:$C,$B41,'BSCR Source Data'!$G:$G,$F41)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A41,'BSCR Aggregated Input'!$C:$C,$B41,'BSCR Aggregated Input'!$G:$G,$F41)</f>
         <v>107224705.2</v>
       </c>
       <c r="D41">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A41,'BSCR Source Data'!$C:$C,$B41,'BSCR Source Data'!$G:$G,$F41)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A41,'BSCR Aggregated Input'!$C:$C,$B41,'BSCR Aggregated Input'!$G:$G,$F41)</f>
         <v>106417749.2</v>
       </c>
       <c r="E41">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A41,'BSCR Source Data'!$C:$C,$B41,'BSCR Source Data'!$G:$G,$F41)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A41,'BSCR Aggregated Input'!$C:$C,$B41,'BSCR Aggregated Input'!$G:$G,$F41)</f>
         <v>86</v>
       </c>
       <c r="F41">
@@ -12303,15 +12327,15 @@
         <v>14</v>
       </c>
       <c r="C42" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A42,'BSCR Source Data'!$C:$C,$B42,'BSCR Source Data'!$G:$G,$F42)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A42,'BSCR Aggregated Input'!$C:$C,$B42,'BSCR Aggregated Input'!$G:$G,$F42)</f>
         <v>2365811503</v>
       </c>
       <c r="D42" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A42,'BSCR Source Data'!$C:$C,$B42,'BSCR Source Data'!$G:$G,$F42)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A42,'BSCR Aggregated Input'!$C:$C,$B42,'BSCR Aggregated Input'!$G:$G,$F42)</f>
         <v>1413295965</v>
       </c>
       <c r="E42">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A42,'BSCR Source Data'!$C:$C,$B42,'BSCR Source Data'!$G:$G,$F42)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A42,'BSCR Aggregated Input'!$C:$C,$B42,'BSCR Aggregated Input'!$G:$G,$F42)</f>
         <v>326</v>
       </c>
       <c r="F42">
@@ -12342,15 +12366,15 @@
         <v>14</v>
       </c>
       <c r="C43" s="1">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A43,'BSCR Source Data'!$C:$C,$B43,'BSCR Source Data'!$G:$G,$F43)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A43,'BSCR Aggregated Input'!$C:$C,$B43,'BSCR Aggregated Input'!$G:$G,$F43)</f>
         <v>738973417.3</v>
       </c>
       <c r="D43" s="1">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A43,'BSCR Source Data'!$C:$C,$B43,'BSCR Source Data'!$G:$G,$F43)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A43,'BSCR Aggregated Input'!$C:$C,$B43,'BSCR Aggregated Input'!$G:$G,$F43)</f>
         <v>426252309.8</v>
       </c>
       <c r="E43">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A43,'BSCR Source Data'!$C:$C,$B43,'BSCR Source Data'!$G:$G,$F43)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A43,'BSCR Aggregated Input'!$C:$C,$B43,'BSCR Aggregated Input'!$G:$G,$F43)</f>
         <v>106</v>
       </c>
       <c r="F43">
@@ -12381,15 +12405,15 @@
         <v>14</v>
       </c>
       <c r="C44">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A44,'BSCR Source Data'!$C:$C,$B44,'BSCR Source Data'!$G:$G,$F44)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A44,'BSCR Aggregated Input'!$C:$C,$B44,'BSCR Aggregated Input'!$G:$G,$F44)</f>
         <v>345000</v>
       </c>
       <c r="D44">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A44,'BSCR Source Data'!$C:$C,$B44,'BSCR Source Data'!$G:$G,$F44)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A44,'BSCR Aggregated Input'!$C:$C,$B44,'BSCR Aggregated Input'!$G:$G,$F44)</f>
         <v>345000</v>
       </c>
       <c r="E44">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A44,'BSCR Source Data'!$C:$C,$B44,'BSCR Source Data'!$G:$G,$F44)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A44,'BSCR Aggregated Input'!$C:$C,$B44,'BSCR Aggregated Input'!$G:$G,$F44)</f>
         <v>1</v>
       </c>
       <c r="F44">
@@ -12420,15 +12444,15 @@
         <v>14</v>
       </c>
       <c r="C45">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A45,'BSCR Source Data'!$C:$C,$B45,'BSCR Source Data'!$G:$G,$F45)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A45,'BSCR Aggregated Input'!$C:$C,$B45,'BSCR Aggregated Input'!$G:$G,$F45)</f>
         <v>2462700</v>
       </c>
       <c r="D45">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A45,'BSCR Source Data'!$C:$C,$B45,'BSCR Source Data'!$G:$G,$F45)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A45,'BSCR Aggregated Input'!$C:$C,$B45,'BSCR Aggregated Input'!$G:$G,$F45)</f>
         <v>2462700</v>
       </c>
       <c r="E45">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A45,'BSCR Source Data'!$C:$C,$B45,'BSCR Source Data'!$G:$G,$F45)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A45,'BSCR Aggregated Input'!$C:$C,$B45,'BSCR Aggregated Input'!$G:$G,$F45)</f>
         <v>3</v>
       </c>
       <c r="F45">
@@ -12459,15 +12483,15 @@
         <v>14</v>
       </c>
       <c r="C46">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A46,'BSCR Source Data'!$C:$C,$B46,'BSCR Source Data'!$G:$G,$F46)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A46,'BSCR Aggregated Input'!$C:$C,$B46,'BSCR Aggregated Input'!$G:$G,$F46)</f>
         <v>101000</v>
       </c>
       <c r="D46">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A46,'BSCR Source Data'!$C:$C,$B46,'BSCR Source Data'!$G:$G,$F46)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A46,'BSCR Aggregated Input'!$C:$C,$B46,'BSCR Aggregated Input'!$G:$G,$F46)</f>
         <v>101000</v>
       </c>
       <c r="E46">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A46,'BSCR Source Data'!$C:$C,$B46,'BSCR Source Data'!$G:$G,$F46)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A46,'BSCR Aggregated Input'!$C:$C,$B46,'BSCR Aggregated Input'!$G:$G,$F46)</f>
         <v>1</v>
       </c>
       <c r="F46">
@@ -12498,15 +12522,15 @@
         <v>14</v>
       </c>
       <c r="C47">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A47,'BSCR Source Data'!$C:$C,$B47,'BSCR Source Data'!$G:$G,$F47)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A47,'BSCR Aggregated Input'!$C:$C,$B47,'BSCR Aggregated Input'!$G:$G,$F47)</f>
         <v>22746034</v>
       </c>
       <c r="D47">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A47,'BSCR Source Data'!$C:$C,$B47,'BSCR Source Data'!$G:$G,$F47)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A47,'BSCR Aggregated Input'!$C:$C,$B47,'BSCR Aggregated Input'!$G:$G,$F47)</f>
         <v>22746034</v>
       </c>
       <c r="E47">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A47,'BSCR Source Data'!$C:$C,$B47,'BSCR Source Data'!$G:$G,$F47)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A47,'BSCR Aggregated Input'!$C:$C,$B47,'BSCR Aggregated Input'!$G:$G,$F47)</f>
         <v>32</v>
       </c>
       <c r="F47">
@@ -12537,15 +12561,15 @@
         <v>14</v>
       </c>
       <c r="C48">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A48,'BSCR Source Data'!$C:$C,$B48,'BSCR Source Data'!$G:$G,$F48)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A48,'BSCR Aggregated Input'!$C:$C,$B48,'BSCR Aggregated Input'!$G:$G,$F48)</f>
         <v>175292598.8</v>
       </c>
       <c r="D48">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A48,'BSCR Source Data'!$C:$C,$B48,'BSCR Source Data'!$G:$G,$F48)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A48,'BSCR Aggregated Input'!$C:$C,$B48,'BSCR Aggregated Input'!$G:$G,$F48)</f>
         <v>87273963.57</v>
       </c>
       <c r="E48">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A48,'BSCR Source Data'!$C:$C,$B48,'BSCR Source Data'!$G:$G,$F48)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A48,'BSCR Aggregated Input'!$C:$C,$B48,'BSCR Aggregated Input'!$G:$G,$F48)</f>
         <v>20</v>
       </c>
       <c r="F48">
@@ -12576,15 +12600,15 @@
         <v>14</v>
       </c>
       <c r="C49">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A49,'BSCR Source Data'!$C:$C,$B49,'BSCR Source Data'!$G:$G,$F49)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A49,'BSCR Aggregated Input'!$C:$C,$B49,'BSCR Aggregated Input'!$G:$G,$F49)</f>
         <v>906507554.6</v>
       </c>
       <c r="D49">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A49,'BSCR Source Data'!$C:$C,$B49,'BSCR Source Data'!$G:$G,$F49)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A49,'BSCR Aggregated Input'!$C:$C,$B49,'BSCR Aggregated Input'!$G:$G,$F49)</f>
         <v>666539312.4</v>
       </c>
       <c r="E49">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A49,'BSCR Source Data'!$C:$C,$B49,'BSCR Source Data'!$G:$G,$F49)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A49,'BSCR Aggregated Input'!$C:$C,$B49,'BSCR Aggregated Input'!$G:$G,$F49)</f>
         <v>227</v>
       </c>
       <c r="F49">
@@ -12615,15 +12639,15 @@
         <v>14</v>
       </c>
       <c r="C50">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A50,'BSCR Source Data'!$C:$C,$B50,'BSCR Source Data'!$G:$G,$F50)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$D:$D,'BSCR Aggregated Input'!$B:$B,$A50,'BSCR Aggregated Input'!$C:$C,$B50,'BSCR Aggregated Input'!$G:$G,$F50)</f>
         <v>101774358.8</v>
       </c>
       <c r="D50">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A50,'BSCR Source Data'!$C:$C,$B50,'BSCR Source Data'!$G:$G,$F50)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$E:$E,'BSCR Aggregated Input'!$B:$B,$A50,'BSCR Aggregated Input'!$C:$C,$B50,'BSCR Aggregated Input'!$G:$G,$F50)</f>
         <v>100967402.8</v>
       </c>
       <c r="E50">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A50,'BSCR Source Data'!$C:$C,$B50,'BSCR Source Data'!$G:$G,$F50)</f>
+        <f>SUMIFS('BSCR Aggregated Input'!$F:$F,'BSCR Aggregated Input'!$B:$B,$A50,'BSCR Aggregated Input'!$C:$C,$B50,'BSCR Aggregated Input'!$G:$G,$F50)</f>
         <v>76</v>
       </c>
       <c r="F50">
@@ -31164,7 +31188,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bscr/BSCR_UKEU.py CSV columns A:G: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded.</t>
+          <t>Generated output/bscr-output.csv columns A:G: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Raw bscr-extract.sql output is a different 8-column contract.</t>
         </is>
       </c>
     </row>
@@ -31176,7 +31200,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Paste the CSV into BSCR Source Data A:G without replacing formula columns. Formulas apply 1.35 GBP/USD and divide by 1,000,000; BSCR Output consolidates and BSCR Pivot Summary presents results.</t>
+          <t>Paste generated bscr-output.csv into BSCR Aggregated Input A:G without replacing formula columns. Formulas apply 1.35 GBP/USD and divide by 1,000,000; BSCR Output Rollup consolidates and BSCR Pivot Summary presents results.</t>
         </is>
       </c>
     </row>
@@ -31200,7 +31224,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Refresh BSCR Output and BSCR Pivot Summary after loading. The checked-in piv is older than BSCR Source Data, so reconcile query, CSV, BSCR Source Data, BSCR Output, BSCR Pivot Summary and final cells before use.</t>
+          <t>Refresh BSCR Output Rollup and BSCR Pivot Summary after loading. The checked-in piv is older than BSCR Aggregated Input, so reconcile query, raw SQL CSV, generated CSV, BSCR Aggregated Input, BSCR Output Rollup, BSCR Pivot Summary and final cells before use.</t>
         </is>
       </c>
     </row>
@@ -31486,11 +31510,11 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -31665,11 +31689,11 @@
         </is>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -31736,11 +31760,11 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_nahu")</f>
         <v>30.8434959</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_nahu")</f>
         <v>30.8434959</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -31756,11 +31780,11 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_na_eq")</f>
         <v>0.2862</v>
       </c>
       <c r="C5" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_na_eq")</f>
         <v>0.2862</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -31776,11 +31800,11 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_eu")</f>
         <v>163747.905595587</v>
       </c>
       <c r="C6" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_eu")</f>
         <v>163747.905595587</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -31796,11 +31820,11 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="C7" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -31816,11 +31840,11 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_jp")</f>
         <v>0.3726</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -31935,27 +31959,27 @@
         </is>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$E:$E,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_us_all")</f>
         <v>33</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_us_all")</f>
         <v>30.8434959</v>
       </c>
       <c r="D4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"is_us_all")</f>
         <v>30.8434959</v>
       </c>
       <c r="E4" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-B4</f>
+        <f>SUMIFS('BSCR Output Rollup'!$E:$E,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")-B4</f>
         <v>173654</v>
       </c>
       <c r="F4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-C4</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")-C4</f>
         <v>164322.324372437</v>
       </c>
       <c r="G4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-D4</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")-D4</f>
         <v>164322.324372437</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -31995,15 +32019,15 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$E:$E,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")</f>
         <v>173687</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$I:$I,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="D8" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output Rollup'!$J:$J,'BSCR Output Rollup'!$A:$A,"HIC",'BSCR Output Rollup'!$B:$B,"ALL")</f>
         <v>164353.167868337</v>
       </c>
       <c r="H8" t="inlineStr">

</xml_diff>

<commit_message>
Document BSCR SQL to Python workflow
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -10540,174 +10540,210 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tab / step</t>
+          <t>Step / tab</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Purpose and action</t>
+          <t>Action</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Raw SQL extract</t>
+          <t>1. Run SQL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bscr-extract.sql produces 8 columns: pml, accgrpid, uwritrname, state, userid1, branchname, cntrycode, is_geocoded. Do not paste this raw SQL CSV directly into the workbook.</t>
+          <t>Run bscr/sql/bscr-extract.sql against the correct EDM database. Set @peril and @policy_type for the required run.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pipeline</t>
+          <t>2. Save the SQL CSV</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Point BSCR_UKEU.py BSCR_INPUT_CSV at the raw SQL CSV. It classifies, applies retentions and writes output/bscr-output.csv.</t>
+          <t>Export the query result as CSV with this exact header order: pml, accgrpid, uwritrname, state, userid1, branchname, cntrycode, is_geocoded. This is the raw 8-column input; do not paste it into this workbook yet.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BSCR Aggregated Input</t>
+          <t>3. Configure Python</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paste generated output/bscr-output.csv into A:G only. Expected headers: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Do not overwrite formula columns H:K.</t>
+          <t>Edit bscr/BSCR_UKEU.py: set BSCR_INPUT_CSV to the raw CSV filename, leave PRA_INPUT_CSV = None for BSCR-only, and set OUTPUT_DIR to a new or empty output folder. Example: BSCR_INPUT_CSV = Path(r"C:\Returns\my BSCR extract.csv").</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>4. Run Python</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>From the reporting/ project folder run: uv run --isolated --locked python bscr/BSCR_UKEU.py. Do not pass script arguments. uvx is not required; uv run uses pyproject.toml and uv.lock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5. Check generated CSV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>The script writes output/bscr-output.csv. Confirm its headers are: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Reconcile ALL-row totals and contributing-row counts to the raw SQL CSV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6. BSCR Aggregated Input</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Paste generated output/bscr-output.csv into A:G only. Do not paste the raw SQL CSV. Do not overwrite formula columns H:K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>7. Refresh roll-up</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Use Formulas &gt; Calculate Now or Ctrl+Alt+F9, then Data &gt; Refresh All.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>BSCR Output Rollup</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Formula-driven roll-up by entity, region/peril and geocoding status. Provides gross/net source values plus USD and USD-million values.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>BSCR Pivot Summary</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
-          <t>Review roll-up of BSCR Output Rollup. After loading data, use Data &gt; Refresh All. Treat this as a review view, not the raw source or final return.</t>
+          <t>Review roll-up of BSCR Output Rollup. Treat this as a review view, not the raw source or final return.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Refresh after paste</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Use Formulas &gt; Calculate Now or Ctrl+Alt+F9, then Data &gt; Refresh All.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Final template</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Open 2026 BSCR - UKEU - HIC.xlsx. Transfer approved values with Paste Special &gt; Values only; preserve template formatting, formulas and validation.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Schedule X(a)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>The workings output does not contain approved EP-curve values, annual average loss, standard deviation or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Schedule X(b)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>The workings output does not contain the insurance EP curve or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Schedule X(c)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Use the compact Schedule X(c) tab as a regional exposure reference: B4:C4 Atlantic Basin Hurricane; B5:C5 North American Earthquake; B6:C6 European Windstorm; B7:C7 Japanese Earthquake; B8:C8 Japanese Typhoon proxy.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Schedule X(c) limitation</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>The final template separates statutory property premium, all-other premium, statutory property limits and all-other limits. The current output is a combined regional total, so do not paste it into one split row without an approved mapping.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Schedule X(f)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Modelability and contract-count classifications are not available from the current BSCR output. Keep those final-template fields pending approved source data.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Control</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
-          <t>Record the source CSV, run date, row count, gross/net totals, FX basis, operator and reviewer before transferring values.</t>
+          <t>Record the source CSV, SQL parameters, run date, row count, gross/net totals, FX basis, operator and reviewer before transferring values.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B18"/>
+  <autoFilter ref="A4:B21"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Document BSCR pivot template transfer map
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -10513,8 +10513,8 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
-    <col min="2" max="2" width="115" customWidth="1"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="118" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10532,7 +10532,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BSCR_Workings.xlsx</t>
+          <t>BSCR_Workings.xlsx; final example: 2026 BSCR - UKEU - HIC.xlsx</t>
         </is>
       </c>
     </row>
@@ -10569,7 +10569,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Export the query result as CSV with this exact header order: pml, accgrpid, uwritrname, state, userid1, branchname, cntrycode, is_geocoded. This is the raw 8-column input; do not paste it into this workbook yet.</t>
+          <t>Export the query result as CSV with exact header order: pml, accgrpid, uwritrname, state, userid1, branchname, cntrycode, is_geocoded. This raw 8-column CSV is not the workbook input.</t>
         </is>
       </c>
     </row>
@@ -10581,7 +10581,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Edit bscr/BSCR_UKEU.py: set BSCR_INPUT_CSV to the raw CSV filename, leave PRA_INPUT_CSV = None for BSCR-only, and set OUTPUT_DIR to a new or empty output folder. Example: BSCR_INPUT_CSV = Path(r"C:\Returns\my BSCR extract.csv").</t>
+          <t>Edit bscr/BSCR_UKEU.py: set BSCR_INPUT_CSV to the raw CSV filename, leave PRA_INPUT_CSV = None for BSCR-only, and set OUTPUT_DIR to a new or empty folder.</t>
         </is>
       </c>
     </row>
@@ -10593,7 +10593,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>From the reporting/ project folder run: uv run --isolated --locked python bscr/BSCR_UKEU.py. Do not pass script arguments. uvx is not required; uv run uses pyproject.toml and uv.lock.</t>
+          <t>From the reporting/ project folder run: uv run --isolated --locked python bscr/BSCR_UKEU.py. No script arguments. uvx is not required.</t>
         </is>
       </c>
     </row>
@@ -10605,7 +10605,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The script writes output/bscr-output.csv. Confirm its headers are: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Reconcile ALL-row totals and contributing-row counts to the raw SQL CSV.</t>
+          <t>Confirm output/bscr-output.csv has: cntrycode, bscr_entity, region, sum_pml, sum_net, count_policies, is_geocoded. Reconcile ALL-row totals and contributing-row counts to the raw SQL CSV.</t>
         </is>
       </c>
     </row>
@@ -10653,20 +10653,31 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Review roll-up of BSCR Output Rollup. Treat this as a review view, not the raw source or final return.</t>
+          <t>Review roll-up of BSCR Output Rollup. Current pivot blocks are A3:J24, A39:I50 and A57:I68. Rows 69:78 are outside the pivot blocks and are not valid output.</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pivot reference rows</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>In the current checked-in snapshot, HIC gross is row 63 (Sum of sum_pml_usd/1m) and HIC net is row 64 (Sum of sum_net_usd/1m). After refreshing, find the HIC and measure labels rather than relying only on row numbers.</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Final template</t>
+          <t>Pivot region columns</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Open 2026 BSCR - UKEU - HIC.xlsx. Transfer approved values with Paste Special &gt; Values only; preserve template formatting, formulas and validation.</t>
+          <t>D = ALL; E = is_eu; F = is_jp; G = is_na_eq; H = is_nahu; I = is_us_all.</t>
         </is>
       </c>
     </row>
@@ -10678,7 +10689,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>The workings output does not contain approved EP-curve values, annual average loss, standard deviation or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
+          <t>No direct pivot paste. Use the HIC ALL total only as a control. X(a) requires EP curves, annual average loss, standard deviation, premiums and modelled/not-modelled splits not produced by this workbook.</t>
         </is>
       </c>
     </row>
@@ -10690,60 +10701,120 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The workings output does not contain the insurance EP curve or premium inputs. Do not populate these final-template cells from this workbook; obtain them from the approved catastrophe-model/premium source.</t>
+          <t>No direct pivot paste. X(b) requires the insurance EP curve and premium inputs not produced by this workbook.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Schedule X(c)</t>
+          <t>X(c) Atlantic Basin Hurricane</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Use the compact Schedule X(c) tab as a regional exposure reference: B4:C4 Atlantic Basin Hurricane; B5:C5 North American Earthquake; B6:C6 European Windstorm; B7:C7 Japanese Earthquake; B8:C8 Japanese Typhoon proxy.</t>
+          <t>Copy BSCR Pivot Summary H63 (gross) and H64 (net) to the example template Schedule X(c) E27 and F27: Total all other statutory limits.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Schedule X(c) limitation</t>
+          <t>X(c) North American Earthquake</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>The final template separates statutory property premium, all-other premium, statutory property limits and all-other limits. The current output is a combined regional total, so do not paste it into one split row without an approved mapping.</t>
+          <t>Copy G63 (gross) and G64 (net) to example Schedule X(c) E49 and F49: Total all other statutory limits.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Schedule X(f)</t>
+          <t>X(c) European Windstorm</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Modelability and contract-count classifications are not available from the current BSCR output. Keep those final-template fields pending approved source data.</t>
+          <t>Copy E63 (gross) and E64 (net) to example Schedule X(c) E71 and F71: Total all other statutory limits.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Control</t>
+          <t>X(c) Japanese Earthquake</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Record the source CSV, SQL parameters, run date, row count, gross/net totals, FX basis, operator and reviewer before transferring values.</t>
+          <t>Copy F63 (gross) and F64 (net) to example Schedule X(c) E93 and F93: Total all other statutory limits.</t>
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>X(c) Japanese Typhoon</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Copy F63/F64 again to example Schedule X(c) E115/F115. This is a Japanese-earthquake-region proxy, not an independent typhoon result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>X(c) premium fields</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Do not copy pivot values into the X(c) premium rows. The pivot contains exposure limits, not statutory premium inputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>X(f) example total</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>If using X(f), compact Schedule X(f) B4:G4 maps to example Schedule X(f) E12:J12 (US count/gross/net, then all-other count/gross/net). Calculate the example total cells K12:M12; do not populate modelability rows 10:11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Transfer method</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>In the final example workbook use Paste Special &gt; Values only. Preserve template formatting, formulas and validation. Record source cell, destination cell, run date and reviewer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Control record</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Keep the raw SQL CSV, SQL parameters, generated bscr-output.csv, workbook version, row counts, gross/net totals, FX basis, operator and reviewer together.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:B21"/>
+  <autoFilter ref="A4:B26"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Move BSCR workflow to multi-peril SQL
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -1,49 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamptonr\projects\rr\reporting\bscr\workbooks\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60094F03-6D36-48AB-969C-C7E4D4C03E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="C:\Users\hamptonr\projects\rr\reporting\bscr\workbooks\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60094F03-6D36-48AB-969C-C7E4D4C03E60}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" activeTab="1" xr2:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" activeTab="1" ns6:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="10" r:id="rId1"/>
-    <sheet name="BSCR Pivot Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="BSCR Output" sheetId="1" r:id="rId3"/>
-    <sheet name="BSCR Source Data" sheetId="3" r:id="rId4"/>
-    <sheet name="AUDIT_SUMMARY" sheetId="4" r:id="rId5"/>
-    <sheet name="Settings" sheetId="5" r:id="rId6"/>
-    <sheet name="Schedule X(a)" sheetId="6" r:id="rId7"/>
-    <sheet name="Schedule X(b)" sheetId="7" r:id="rId8"/>
-    <sheet name="Schedule X(c)" sheetId="8" r:id="rId9"/>
-    <sheet name="Schedule X(f)" sheetId="9" r:id="rId10"/>
+    <sheet name="Instructions" sheetId="10" ns7:id="rId1"/>
+    <sheet name="BSCR Pivot Summary" sheetId="2" ns7:id="rId2"/>
+    <sheet name="BSCR Output" sheetId="1" ns7:id="rId3"/>
+    <sheet name="BSCR Source Data" sheetId="3" ns7:id="rId4"/>
+    <sheet name="AUDIT_SUMMARY" sheetId="4" ns7:id="rId5"/>
+    <sheet name="Settings" sheetId="5" ns7:id="rId6"/>
+    <sheet name="Schedule X(a)" sheetId="6" ns7:id="rId7"/>
+    <sheet name="Schedule X(b)" sheetId="7" ns7:id="rId8"/>
+    <sheet name="Schedule X(c)" sheetId="8" ns7:id="rId9"/>
+    <sheet name="Schedule X(f)" sheetId="9" ns7:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BSCR Source Data'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BSCR Output'!$A$1:$F$50</definedName>
   </definedNames>
-  <calcPr calcId="191029" forceFullCalc="1"/>
+  <calcPr calcId="191029" forceFullCalc="1" calcMode="auto" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache cacheId="41" r:id="rId11"/>
-    <pivotCache cacheId="65" r:id="rId12"/>
+    <pivotCache cacheId="41" ns7:id="rId11"/>
+    <pivotCache cacheId="65" ns7:id="rId12"/>
   </pivotCaches>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns8:calcFeatures>
+        <ns8:feature name="microsoft.com:RD"/>
+        <ns8:feature name="microsoft.com:Single"/>
+        <ns8:feature name="microsoft.com:FV"/>
+        <ns8:feature name="microsoft.com:CNMTM"/>
+        <ns8:feature name="microsoft.com:LET_WF"/>
+        <ns8:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns8:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns8:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -10265,20 +10265,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="115" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ns3:dyDescent="0.25">
       <c r="A1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ns3:dyDescent="0.25">
       <c r="A2" t="s">
         <v>140</v>
       </c>
@@ -10286,7 +10286,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ns3:dyDescent="0.25">
       <c r="A4" t="s">
         <v>142</v>
       </c>
@@ -10294,7 +10294,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>144</v>
       </c>
@@ -10302,7 +10302,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ns3:dyDescent="0.25">
       <c r="A6" t="s">
         <v>146</v>
       </c>
@@ -10310,7 +10310,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ns3:dyDescent="0.25">
       <c r="A7" t="s">
         <v>148</v>
       </c>
@@ -10318,7 +10318,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ns3:dyDescent="0.25">
       <c r="A8" t="s">
         <v>150</v>
       </c>
@@ -10326,15 +10326,17 @@
         <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="13" ns3:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B10" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Set Settings!B7 to the entity, refresh the SQL/Power Query source, then review the linked schedules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ns3:dyDescent="0.25">
       <c r="A11" t="s">
         <v>154</v>
       </c>
@@ -10342,7 +10344,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ns3:dyDescent="0.25">
       <c r="A12" t="s">
         <v>155</v>
       </c>
@@ -10350,7 +10352,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ns3:dyDescent="0.25">
       <c r="A13" t="s">
         <v>156</v>
       </c>
@@ -10358,7 +10360,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ns3:dyDescent="0.25">
       <c r="A14" t="s">
         <v>158</v>
       </c>
@@ -10366,7 +10368,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ns3:dyDescent="0.25">
       <c r="A15" t="s">
         <v>160</v>
       </c>
@@ -10374,7 +10376,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ns3:dyDescent="0.25">
       <c r="A16" t="s">
         <v>162</v>
       </c>
@@ -10383,15 +10385,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B16" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:B16" ns2:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -10402,17 +10404,17 @@
     <col min="8" max="8" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ns3:dyDescent="0.25">
       <c r="A2" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ns3:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>231</v>
       </c>
@@ -10438,39 +10440,39 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ns3:dyDescent="0.25">
       <c r="A4" t="s">
         <v>238</v>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>33</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="D4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="E4" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-B4</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")-B4</f>
         <v>173654</v>
       </c>
       <c r="F4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-C4</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")-C4</f>
         <v>164322.32437243802</v>
       </c>
       <c r="G4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-D4</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")-D4</f>
         <v>164322.32437243802</v>
       </c>
       <c r="H4" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>240</v>
       </c>
@@ -10478,7 +10480,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ns3:dyDescent="0.25">
       <c r="A6" t="s">
         <v>242</v>
       </c>
@@ -10486,20 +10488,20 @@
         <v>241</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ns3:dyDescent="0.25">
       <c r="A8" t="s">
         <v>243</v>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
         <v>173687</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="D8" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="H8" t="s">
@@ -11979,9 +11981,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD6788F1-4B47-421A-9EF9-440A877182E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{FD6788F1-4B47-421A-9EF9-440A877182E4}">
   <dimension ref="A1:J82"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.453125" style="14" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7265625" style="12"/>
@@ -11994,7 +11996,7 @@
     <col min="10" max="10" width="16.54296875" style="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ns3:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -12026,7 +12028,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ns3:dyDescent="0.25">
       <c r="A2" s="14">
         <v>33</v>
       </c>
@@ -12065,7 +12067,7 @@
         <v>3958.1360793249482</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ns3:dyDescent="0.25">
       <c r="A3" s="14">
         <v>33</v>
       </c>
@@ -12104,7 +12106,7 @@
         <v>25145.813471997968</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ns3:dyDescent="0.25">
       <c r="A4" s="14">
         <v>3624</v>
       </c>
@@ -12143,7 +12145,7 @@
         <v>2.2302</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ns3:dyDescent="0.25">
       <c r="A5" s="14">
         <v>3624</v>
       </c>
@@ -12182,7 +12184,7 @@
         <v>27.559570680000004</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ns3:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>7</v>
       </c>
@@ -12221,7 +12223,7 @@
         <v>20.835638639999999</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ns3:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>7</v>
       </c>
@@ -12260,7 +12262,7 @@
         <v>164332.33222969799</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ns3:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>8</v>
       </c>
@@ -12299,7 +12301,7 @@
         <v>549.39890388437016</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ns3:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>8</v>
       </c>
@@ -12338,7 +12340,7 @@
         <v>7872.8932494682404</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ns3:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>9</v>
       </c>
@@ -12377,7 +12379,7 @@
         <v>471.54302374525707</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ns3:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>9</v>
       </c>
@@ -12416,7 +12418,7 @@
         <v>101945.66631185531</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ns3:dyDescent="0.25">
       <c r="A12" s="14">
         <v>33</v>
       </c>
@@ -12455,7 +12457,7 @@
         <v>533.79541228629068</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ns3:dyDescent="0.25">
       <c r="A13" s="14">
         <v>33</v>
       </c>
@@ -12494,7 +12496,7 @@
         <v>16379.079800502455</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ns3:dyDescent="0.25">
       <c r="A14" s="14">
         <v>3624</v>
       </c>
@@ -12533,7 +12535,7 @@
         <v>7.5303000000000013</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ns3:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>7</v>
       </c>
@@ -12572,7 +12574,7 @@
         <v>9.5849271000000016</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ns3:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>7</v>
       </c>
@@ -12611,7 +12613,7 @@
         <v>163738.32066848699</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ns3:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>8</v>
       </c>
@@ -12650,7 +12652,7 @@
         <v>152.02980438751484</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ns3:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>8</v>
       </c>
@@ -12689,7 +12691,7 @@
         <v>2961.399227134893</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ns3:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>9</v>
       </c>
@@ -12728,7 +12730,7 @@
         <v>101.89685250025703</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ns3:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>9</v>
       </c>
@@ -12767,7 +12769,7 @@
         <v>73898.852478824294</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ns3:dyDescent="0.25">
       <c r="A21" s="14">
         <v>33</v>
       </c>
@@ -12806,7 +12808,7 @@
         <v>2.1592000809639047</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ns3:dyDescent="0.25">
       <c r="A22" s="14">
         <v>33</v>
       </c>
@@ -12845,7 +12847,7 @@
         <v>64.189409847055387</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ns3:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>7</v>
       </c>
@@ -12884,7 +12886,7 @@
         <v>0.37259999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ns3:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>8</v>
       </c>
@@ -12923,7 +12925,7 @@
         <v>144.49731873975227</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ns3:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>9</v>
       </c>
@@ -12962,7 +12964,7 @@
         <v>27.271459080000003</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ns3:dyDescent="0.25">
       <c r="A26" s="14">
         <v>33</v>
       </c>
@@ -13001,7 +13003,7 @@
         <v>22.247616184646581</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ns3:dyDescent="0.25">
       <c r="A27" s="14">
         <v>33</v>
       </c>
@@ -13040,7 +13042,7 @@
         <v>143.9522816275782</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ns3:dyDescent="0.25">
       <c r="A28" s="14">
         <v>3624</v>
       </c>
@@ -13079,7 +13081,7 @@
         <v>0.14849999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ns3:dyDescent="0.25">
       <c r="A29" s="14">
         <v>3624</v>
       </c>
@@ -13118,7 +13120,7 @@
         <v>0.14849999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ns3:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>7</v>
       </c>
@@ -13157,7 +13159,7 @@
         <v>0.28620000000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ns3:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>8</v>
       </c>
@@ -13196,7 +13198,7 @@
         <v>10.203767316443908</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ns3:dyDescent="0.25">
       <c r="A32" s="14" t="s">
         <v>9</v>
       </c>
@@ -13235,7 +13237,7 @@
         <v>0.75600000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ns3:dyDescent="0.25">
       <c r="A33" s="14">
         <v>33</v>
       </c>
@@ -13274,7 +13276,7 @@
         <v>1917.5542448334215</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ns3:dyDescent="0.25">
       <c r="A34" s="14">
         <v>33</v>
       </c>
@@ -13313,7 +13315,7 @@
         <v>606.07039780486548</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ns3:dyDescent="0.25">
       <c r="A35" s="14">
         <v>3624</v>
       </c>
@@ -13352,7 +13354,7 @@
         <v>0.73575000000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ns3:dyDescent="0.25">
       <c r="A36" s="14">
         <v>3624</v>
       </c>
@@ -13391,7 +13393,7 @@
         <v>3.5946450000000003</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ns3:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>7</v>
       </c>
@@ -13430,7 +13432,7 @@
         <v>0.13635</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ns3:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>7</v>
       </c>
@@ -13469,7 +13471,7 @@
         <v>30.707145900000004</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" ns3:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>8</v>
       </c>
@@ -13508,7 +13510,7 @@
         <v>140.02584614885711</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" ns3:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>8</v>
       </c>
@@ -13547,7 +13549,7 @@
         <v>1248.0576953635141</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" ns3:dyDescent="0.25">
       <c r="A41" s="14" t="s">
         <v>9</v>
       </c>
@@ -13586,7 +13588,7 @@
         <v>143.66396144153524</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" ns3:dyDescent="0.25">
       <c r="A42" s="14">
         <v>33</v>
       </c>
@@ -13625,7 +13627,7 @@
         <v>1907.9495532296821</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" ns3:dyDescent="0.25">
       <c r="A43" s="14">
         <v>33</v>
       </c>
@@ -13664,7 +13666,7 @@
         <v>575.44061825384767</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" ns3:dyDescent="0.25">
       <c r="A44" s="14">
         <v>3624</v>
       </c>
@@ -13703,7 +13705,7 @@
         <v>0.46575000000000005</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" ns3:dyDescent="0.25">
       <c r="A45" s="14">
         <v>3624</v>
       </c>
@@ -13742,7 +13744,7 @@
         <v>3.3246449999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" ns3:dyDescent="0.25">
       <c r="A46" s="14" t="s">
         <v>7</v>
       </c>
@@ -13781,7 +13783,7 @@
         <v>0.13635</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" ns3:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>7</v>
       </c>
@@ -13820,7 +13822,7 @@
         <v>30.707145900000004</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" ns3:dyDescent="0.25">
       <c r="A48" s="14" t="s">
         <v>8</v>
       </c>
@@ -13859,7 +13861,7 @@
         <v>117.81985081837681</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" ns3:dyDescent="0.25">
       <c r="A49" s="14" t="s">
         <v>8</v>
       </c>
@@ -13898,7 +13900,7 @@
         <v>899.82807173966796</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" ns3:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>9</v>
       </c>
@@ -13937,131 +13939,911 @@
         <v>136.30599380153521</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I51" s="16"/>
-      <c r="J51" s="16"/>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I52" s="16"/>
-      <c r="J52" s="16"/>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I53" s="16"/>
-      <c r="J53" s="16"/>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I54" s="16"/>
-      <c r="J54" s="16"/>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I55" s="16"/>
-      <c r="J55" s="16"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I56" s="16"/>
-      <c r="J56" s="16"/>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I57" s="16"/>
-      <c r="J57" s="16"/>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I58" s="16"/>
-      <c r="J58" s="16"/>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I59" s="16"/>
-      <c r="J59" s="16"/>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I60" s="16"/>
-      <c r="J60" s="16"/>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I61" s="16"/>
-      <c r="J61" s="16"/>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I62" s="16"/>
-      <c r="J62" s="16"/>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I63" s="16"/>
-      <c r="J63" s="16"/>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="I64" s="16"/>
-      <c r="J64" s="16"/>
-    </row>
-    <row r="65" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I65" s="16"/>
-      <c r="J65" s="16"/>
-    </row>
-    <row r="66" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I66" s="16"/>
-      <c r="J66" s="16"/>
-    </row>
-    <row r="67" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I67" s="16"/>
-      <c r="J67" s="16"/>
-    </row>
-    <row r="68" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I68" s="16"/>
-      <c r="J68" s="16"/>
-    </row>
-    <row r="69" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I69" s="16"/>
-      <c r="J69" s="16"/>
-    </row>
-    <row r="70" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I70" s="16"/>
-      <c r="J70" s="16"/>
-    </row>
-    <row r="71" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C51" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A51,'BSCR Source Data'!$C:$C,$B51,'BSCR Source Data'!$G:$G,$F51)</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A51,'BSCR Source Data'!$C:$C,$B51,'BSCR Source Data'!$G:$G,$F51)</f>
+        <v>0</v>
+      </c>
+      <c r="E51" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A51,'BSCR Source Data'!$C:$C,$B51,'BSCR Source Data'!$G:$G,$F51)</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="12">
+        <v>0</v>
+      </c>
+      <c r="G51" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H51" s="15">
+        <f>D51*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J51" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C52" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A52,'BSCR Source Data'!$C:$C,$B52,'BSCR Source Data'!$G:$G,$F52)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A52,'BSCR Source Data'!$C:$C,$B52,'BSCR Source Data'!$G:$G,$F52)</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A52,'BSCR Source Data'!$C:$C,$B52,'BSCR Source Data'!$G:$G,$F52)</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="12">
+        <v>1</v>
+      </c>
+      <c r="G52" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H52" s="15">
+        <f>D52*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I52" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J52" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>3624</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C53" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A53,'BSCR Source Data'!$C:$C,$B53,'BSCR Source Data'!$G:$G,$F53)</f>
+        <v>0</v>
+      </c>
+      <c r="D53" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A53,'BSCR Source Data'!$C:$C,$B53,'BSCR Source Data'!$G:$G,$F53)</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A53,'BSCR Source Data'!$C:$C,$B53,'BSCR Source Data'!$G:$G,$F53)</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="12">
+        <v>0</v>
+      </c>
+      <c r="G53" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H53" s="15">
+        <f>D53*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J53" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>3624</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C54" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A54,'BSCR Source Data'!$C:$C,$B54,'BSCR Source Data'!$G:$G,$F54)</f>
+        <v>0</v>
+      </c>
+      <c r="D54" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A54,'BSCR Source Data'!$C:$C,$B54,'BSCR Source Data'!$G:$G,$F54)</f>
+        <v>0</v>
+      </c>
+      <c r="E54" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A54,'BSCR Source Data'!$C:$C,$B54,'BSCR Source Data'!$G:$G,$F54)</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="12">
+        <v>1</v>
+      </c>
+      <c r="G54" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H54" s="15">
+        <f>D54*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I54" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J54" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>HIC</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C55" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A55,'BSCR Source Data'!$C:$C,$B55,'BSCR Source Data'!$G:$G,$F55)</f>
+        <v>0</v>
+      </c>
+      <c r="D55" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A55,'BSCR Source Data'!$C:$C,$B55,'BSCR Source Data'!$G:$G,$F55)</f>
+        <v>0</v>
+      </c>
+      <c r="E55" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A55,'BSCR Source Data'!$C:$C,$B55,'BSCR Source Data'!$G:$G,$F55)</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="12">
+        <v>0</v>
+      </c>
+      <c r="G55" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H55" s="15">
+        <f>D55*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I55" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J55" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>HIC</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C56" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A56,'BSCR Source Data'!$C:$C,$B56,'BSCR Source Data'!$G:$G,$F56)</f>
+        <v>0</v>
+      </c>
+      <c r="D56" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A56,'BSCR Source Data'!$C:$C,$B56,'BSCR Source Data'!$G:$G,$F56)</f>
+        <v>0</v>
+      </c>
+      <c r="E56" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A56,'BSCR Source Data'!$C:$C,$B56,'BSCR Source Data'!$G:$G,$F56)</f>
+        <v>0</v>
+      </c>
+      <c r="F56" s="12">
+        <v>1</v>
+      </c>
+      <c r="G56" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H56" s="15">
+        <f>D56*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I56" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J56" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>HIG</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C57" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A57,'BSCR Source Data'!$C:$C,$B57,'BSCR Source Data'!$G:$G,$F57)</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A57,'BSCR Source Data'!$C:$C,$B57,'BSCR Source Data'!$G:$G,$F57)</f>
+        <v>0</v>
+      </c>
+      <c r="E57" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A57,'BSCR Source Data'!$C:$C,$B57,'BSCR Source Data'!$G:$G,$F57)</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="12">
+        <v>0</v>
+      </c>
+      <c r="G57" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H57" s="15">
+        <f>D57*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I57" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J57" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>HIG</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C58" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A58,'BSCR Source Data'!$C:$C,$B58,'BSCR Source Data'!$G:$G,$F58)</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A58,'BSCR Source Data'!$C:$C,$B58,'BSCR Source Data'!$G:$G,$F58)</f>
+        <v>0</v>
+      </c>
+      <c r="E58" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A58,'BSCR Source Data'!$C:$C,$B58,'BSCR Source Data'!$G:$G,$F58)</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="12">
+        <v>1</v>
+      </c>
+      <c r="G58" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H58" s="15">
+        <f>D58*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I58" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J58" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A59" s="14" t="inlineStr">
+        <is>
+          <t>HSA</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C59" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A59,'BSCR Source Data'!$C:$C,$B59,'BSCR Source Data'!$G:$G,$F59)</f>
+        <v>0</v>
+      </c>
+      <c r="D59" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A59,'BSCR Source Data'!$C:$C,$B59,'BSCR Source Data'!$G:$G,$F59)</f>
+        <v>0</v>
+      </c>
+      <c r="E59" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A59,'BSCR Source Data'!$C:$C,$B59,'BSCR Source Data'!$G:$G,$F59)</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="12">
+        <v>0</v>
+      </c>
+      <c r="G59" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H59" s="15">
+        <f>D59*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I59" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J59" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>HSA</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>is_jp_eq</t>
+        </is>
+      </c>
+      <c r="C60" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A60,'BSCR Source Data'!$C:$C,$B60,'BSCR Source Data'!$G:$G,$F60)</f>
+        <v>0</v>
+      </c>
+      <c r="D60" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A60,'BSCR Source Data'!$C:$C,$B60,'BSCR Source Data'!$G:$G,$F60)</f>
+        <v>0</v>
+      </c>
+      <c r="E60" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A60,'BSCR Source Data'!$C:$C,$B60,'BSCR Source Data'!$G:$G,$F60)</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="12">
+        <v>1</v>
+      </c>
+      <c r="G60" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H60" s="15">
+        <f>D60*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I60" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J60" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C61" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A61,'BSCR Source Data'!$C:$C,$B61,'BSCR Source Data'!$G:$G,$F61)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A61,'BSCR Source Data'!$C:$C,$B61,'BSCR Source Data'!$G:$G,$F61)</f>
+        <v>0</v>
+      </c>
+      <c r="E61" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A61,'BSCR Source Data'!$C:$C,$B61,'BSCR Source Data'!$G:$G,$F61)</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="12">
+        <v>0</v>
+      </c>
+      <c r="G61" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H61" s="15">
+        <f>D61*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I61" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J61" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C62" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A62,'BSCR Source Data'!$C:$C,$B62,'BSCR Source Data'!$G:$G,$F62)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A62,'BSCR Source Data'!$C:$C,$B62,'BSCR Source Data'!$G:$G,$F62)</f>
+        <v>0</v>
+      </c>
+      <c r="E62" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A62,'BSCR Source Data'!$C:$C,$B62,'BSCR Source Data'!$G:$G,$F62)</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="12">
+        <v>1</v>
+      </c>
+      <c r="G62" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H62" s="15">
+        <f>D62*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I62" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J62" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>3624</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C63" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A63,'BSCR Source Data'!$C:$C,$B63,'BSCR Source Data'!$G:$G,$F63)</f>
+        <v>0</v>
+      </c>
+      <c r="D63" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A63,'BSCR Source Data'!$C:$C,$B63,'BSCR Source Data'!$G:$G,$F63)</f>
+        <v>0</v>
+      </c>
+      <c r="E63" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A63,'BSCR Source Data'!$C:$C,$B63,'BSCR Source Data'!$G:$G,$F63)</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="12">
+        <v>0</v>
+      </c>
+      <c r="G63" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H63" s="15">
+        <f>D63*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I63" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J63" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>3624</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C64" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A64,'BSCR Source Data'!$C:$C,$B64,'BSCR Source Data'!$G:$G,$F64)</f>
+        <v>0</v>
+      </c>
+      <c r="D64" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A64,'BSCR Source Data'!$C:$C,$B64,'BSCR Source Data'!$G:$G,$F64)</f>
+        <v>0</v>
+      </c>
+      <c r="E64" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A64,'BSCR Source Data'!$C:$C,$B64,'BSCR Source Data'!$G:$G,$F64)</f>
+        <v>0</v>
+      </c>
+      <c r="F64" s="12">
+        <v>1</v>
+      </c>
+      <c r="G64" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H64" s="15">
+        <f>D64*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I64" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J64" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t>HIC</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C65" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A65,'BSCR Source Data'!$C:$C,$B65,'BSCR Source Data'!$G:$G,$F65)</f>
+        <v>0</v>
+      </c>
+      <c r="D65" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A65,'BSCR Source Data'!$C:$C,$B65,'BSCR Source Data'!$G:$G,$F65)</f>
+        <v>0</v>
+      </c>
+      <c r="E65" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A65,'BSCR Source Data'!$C:$C,$B65,'BSCR Source Data'!$G:$G,$F65)</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="12">
+        <v>0</v>
+      </c>
+      <c r="G65" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H65" s="15">
+        <f>D65*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I65" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J65" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>HIC</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C66" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A66,'BSCR Source Data'!$C:$C,$B66,'BSCR Source Data'!$G:$G,$F66)</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A66,'BSCR Source Data'!$C:$C,$B66,'BSCR Source Data'!$G:$G,$F66)</f>
+        <v>0</v>
+      </c>
+      <c r="E66" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A66,'BSCR Source Data'!$C:$C,$B66,'BSCR Source Data'!$G:$G,$F66)</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="12">
+        <v>1</v>
+      </c>
+      <c r="G66" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H66" s="15">
+        <f>D66*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I66" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J66" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A67" s="14" t="inlineStr">
+        <is>
+          <t>HIG</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C67" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A67,'BSCR Source Data'!$C:$C,$B67,'BSCR Source Data'!$G:$G,$F67)</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A67,'BSCR Source Data'!$C:$C,$B67,'BSCR Source Data'!$G:$G,$F67)</f>
+        <v>0</v>
+      </c>
+      <c r="E67" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A67,'BSCR Source Data'!$C:$C,$B67,'BSCR Source Data'!$G:$G,$F67)</f>
+        <v>0</v>
+      </c>
+      <c r="F67" s="12">
+        <v>0</v>
+      </c>
+      <c r="G67" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H67" s="15">
+        <f>D67*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I67" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J67" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>HIG</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C68" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A68,'BSCR Source Data'!$C:$C,$B68,'BSCR Source Data'!$G:$G,$F68)</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A68,'BSCR Source Data'!$C:$C,$B68,'BSCR Source Data'!$G:$G,$F68)</f>
+        <v>0</v>
+      </c>
+      <c r="E68" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A68,'BSCR Source Data'!$C:$C,$B68,'BSCR Source Data'!$G:$G,$F68)</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="12">
+        <v>1</v>
+      </c>
+      <c r="G68" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H68" s="15">
+        <f>D68*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I68" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J68" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>HSA</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C69" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A69,'BSCR Source Data'!$C:$C,$B69,'BSCR Source Data'!$G:$G,$F69)</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A69,'BSCR Source Data'!$C:$C,$B69,'BSCR Source Data'!$G:$G,$F69)</f>
+        <v>0</v>
+      </c>
+      <c r="E69" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A69,'BSCR Source Data'!$C:$C,$B69,'BSCR Source Data'!$G:$G,$F69)</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="12">
+        <v>0</v>
+      </c>
+      <c r="G69" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H69" s="15">
+        <f>D69*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I69" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J69" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ns3:dyDescent="0.25">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>HSA</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>is_non_us</t>
+        </is>
+      </c>
+      <c r="C70" s="12">
+        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A70,'BSCR Source Data'!$C:$C,$B70,'BSCR Source Data'!$G:$G,$F70)</f>
+        <v>0</v>
+      </c>
+      <c r="D70" s="12">
+        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A70,'BSCR Source Data'!$C:$C,$B70,'BSCR Source Data'!$G:$G,$F70)</f>
+        <v>0</v>
+      </c>
+      <c r="E70" s="12">
+        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A70,'BSCR Source Data'!$C:$C,$B70,'BSCR Source Data'!$G:$G,$F70)</f>
+        <v>0</v>
+      </c>
+      <c r="F70" s="12">
+        <v>1</v>
+      </c>
+      <c r="G70" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H70" s="15">
+        <f>D70*Settings!$B$3</f>
+        <v>0</v>
+      </c>
+      <c r="I70" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J70" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="9:10" ns3:dyDescent="0.25">
       <c r="I71" s="16"/>
       <c r="J71" s="16"/>
     </row>
-    <row r="72" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="9:10" ns3:dyDescent="0.25">
       <c r="I72" s="16"/>
       <c r="J72" s="16"/>
     </row>
-    <row r="73" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="9:10" ns3:dyDescent="0.25">
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
     </row>
-    <row r="74" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="9:10" ns3:dyDescent="0.25">
       <c r="I74" s="16"/>
       <c r="J74" s="16"/>
     </row>
-    <row r="75" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="9:10" ns3:dyDescent="0.25">
       <c r="I75" s="16"/>
       <c r="J75" s="16"/>
     </row>
-    <row r="76" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="9:10" ns3:dyDescent="0.25">
       <c r="I76" s="16"/>
       <c r="J76" s="16"/>
     </row>
-    <row r="77" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="9:10" ns3:dyDescent="0.25">
       <c r="I77" s="16"/>
       <c r="J77" s="16"/>
     </row>
-    <row r="78" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="9:10" ns3:dyDescent="0.25">
       <c r="I78" s="16"/>
       <c r="J78" s="16"/>
     </row>
-    <row r="79" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="9:10" ns3:dyDescent="0.25">
       <c r="I79" s="16"/>
       <c r="J79" s="16"/>
     </row>
-    <row r="80" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="9:10" ns3:dyDescent="0.25">
       <c r="I80" s="16"/>
       <c r="J80" s="16"/>
     </row>
-    <row r="81" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="9:10" ns3:dyDescent="0.25">
       <c r="I81" s="16"/>
       <c r="J81" s="16"/>
     </row>
-    <row r="82" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="9:10" ns3:dyDescent="0.25">
       <c r="I82" s="16"/>
       <c r="J82" s="16"/>
     </row>
@@ -32310,9 +33092,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -32320,12 +33102,12 @@
     <col min="4" max="4" width="82" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ns3:dyDescent="0.25">
       <c r="A3" t="s">
         <v>184</v>
       </c>
@@ -32333,7 +33115,7 @@
         <v>1.35</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ns3:dyDescent="0.25">
       <c r="A4" t="s">
         <v>185</v>
       </c>
@@ -32341,7 +33123,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>187</v>
       </c>
@@ -32349,7 +33131,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ns3:dyDescent="0.25">
       <c r="A6" t="s">
         <v>189</v>
       </c>
@@ -32357,7 +33139,19 @@
         <v>190</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ns3:dyDescent="0.25">
       <c r="A8" t="s">
         <v>191</v>
       </c>
@@ -32366,31 +33160,36 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="0" sqref="B7">
+      <formula1>"33,HIC,HIG,HSA,3624"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.3" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ns3:dyDescent="0.25">
       <c r="A2" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ns3:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>195</v>
       </c>
@@ -32404,7 +33203,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ns3:dyDescent="0.25">
       <c r="A4" t="s">
         <v>198</v>
       </c>
@@ -32412,7 +33211,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>200</v>
       </c>
@@ -32420,7 +33219,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ns3:dyDescent="0.25">
       <c r="A6" t="s">
         <v>201</v>
       </c>
@@ -32428,7 +33227,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ns3:dyDescent="0.25">
       <c r="A7" t="s">
         <v>202</v>
       </c>
@@ -32436,7 +33235,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ns3:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -32444,7 +33243,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ns3:dyDescent="0.25">
       <c r="A9" t="s">
         <v>204</v>
       </c>
@@ -32452,7 +33251,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ns3:dyDescent="0.25">
       <c r="A10" t="s">
         <v>205</v>
       </c>
@@ -32460,7 +33259,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ns3:dyDescent="0.25">
       <c r="A11" t="s">
         <v>206</v>
       </c>
@@ -32468,7 +33267,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ns3:dyDescent="0.25">
       <c r="A12" t="s">
         <v>207</v>
       </c>
@@ -32476,16 +33275,16 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ns3:dyDescent="0.25">
       <c r="A14" t="s">
         <v>208</v>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="D14" t="s">
@@ -32498,26 +33297,26 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ns3:dyDescent="0.25">
       <c r="A2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ns3:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>195</v>
       </c>
@@ -32531,7 +33330,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ns3:dyDescent="0.25">
       <c r="A4" t="s">
         <v>198</v>
       </c>
@@ -32539,7 +33338,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>200</v>
       </c>
@@ -32547,7 +33346,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ns3:dyDescent="0.25">
       <c r="A6" t="s">
         <v>201</v>
       </c>
@@ -32555,7 +33354,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ns3:dyDescent="0.25">
       <c r="A7" t="s">
         <v>202</v>
       </c>
@@ -32563,7 +33362,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ns3:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -32571,7 +33370,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ns3:dyDescent="0.25">
       <c r="A9" t="s">
         <v>204</v>
       </c>
@@ -32579,7 +33378,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ns3:dyDescent="0.25">
       <c r="A10" t="s">
         <v>205</v>
       </c>
@@ -32587,7 +33386,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ns3:dyDescent="0.25">
       <c r="A11" t="s">
         <v>206</v>
       </c>
@@ -32595,7 +33394,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ns3:dyDescent="0.25">
       <c r="A12" t="s">
         <v>207</v>
       </c>
@@ -32603,16 +33402,16 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ns3:dyDescent="0.25">
       <c r="A14" t="s">
         <v>208</v>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="D14" t="s">
@@ -32625,26 +33424,26 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ns3:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ns3:dyDescent="0.25">
       <c r="A2" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ns3:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>214</v>
       </c>
@@ -32658,87 +33457,87 @@
         <v>217</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ns3:dyDescent="0.25">
       <c r="A4" t="s">
         <v>218</v>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_nahu")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_nahu")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="D4" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ns3:dyDescent="0.25">
       <c r="A5" t="s">
         <v>220</v>
       </c>
       <c r="B5" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_na_eq")</f>
         <v>0.28620000000000001</v>
       </c>
       <c r="C5" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_na_eq")</f>
         <v>0.28620000000000001</v>
       </c>
       <c r="D5" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ns3:dyDescent="0.25">
       <c r="A6" t="s">
         <v>221</v>
       </c>
       <c r="B6" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_eu")</f>
         <v>163747.90559558698</v>
       </c>
       <c r="C6" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_eu")</f>
         <v>163747.90559558698</v>
       </c>
       <c r="D6" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ns3:dyDescent="0.25">
       <c r="A7" t="s">
         <v>222</v>
       </c>
       <c r="B7" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="C7" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="D7" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ns3:dyDescent="0.25">
       <c r="A8" t="s">
         <v>223</v>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp_eq")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp_eq")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="D8" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ns3:dyDescent="0.25">
       <c r="A11" t="s">
         <v>225</v>
       </c>
@@ -32746,7 +33545,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ns3:dyDescent="0.25">
       <c r="A12" t="s">
         <v>227</v>
       </c>

</xml_diff>

<commit_message>
Restore earlier BSCR workings and archive historical Python entrypoints
</commit_message>
<xml_diff>
--- a/reporting/bscr/workbooks/BSCR_Workings.xlsx
+++ b/reporting/bscr/workbooks/BSCR_Workings.xlsx
@@ -1,49 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns7="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <ns1:AlternateContent>
-    <ns1:Choice Requires="x15">
-      <ns2:absPath url="C:\Users\hamptonr\projects\rr\reporting\bscr\workbooks\"/>
-    </ns1:Choice>
-  </ns1:AlternateContent>
-  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60094F03-6D36-48AB-969C-C7E4D4C03E60}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamptonr\projects\rr\reporting\bscr\workbooks\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60094F03-6D36-48AB-969C-C7E4D4C03E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" activeTab="1" ns6:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" activeTab="1" xr2:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="10" ns7:id="rId1"/>
-    <sheet name="BSCR Pivot Summary" sheetId="2" ns7:id="rId2"/>
-    <sheet name="BSCR Output" sheetId="1" ns7:id="rId3"/>
-    <sheet name="BSCR Source Data" sheetId="3" ns7:id="rId4"/>
-    <sheet name="AUDIT_SUMMARY" sheetId="4" ns7:id="rId5"/>
-    <sheet name="Settings" sheetId="5" ns7:id="rId6"/>
-    <sheet name="Schedule X(a)" sheetId="6" ns7:id="rId7"/>
-    <sheet name="Schedule X(b)" sheetId="7" ns7:id="rId8"/>
-    <sheet name="Schedule X(c)" sheetId="8" ns7:id="rId9"/>
-    <sheet name="Schedule X(f)" sheetId="9" ns7:id="rId10"/>
+    <sheet name="Instructions" sheetId="10" r:id="rId1"/>
+    <sheet name="BSCR Pivot Summary" sheetId="2" r:id="rId2"/>
+    <sheet name="BSCR Output" sheetId="1" r:id="rId3"/>
+    <sheet name="BSCR Source Data" sheetId="3" r:id="rId4"/>
+    <sheet name="AUDIT_SUMMARY" sheetId="4" r:id="rId5"/>
+    <sheet name="Settings" sheetId="5" r:id="rId6"/>
+    <sheet name="Schedule X(a)" sheetId="6" r:id="rId7"/>
+    <sheet name="Schedule X(b)" sheetId="7" r:id="rId8"/>
+    <sheet name="Schedule X(c)" sheetId="8" r:id="rId9"/>
+    <sheet name="Schedule X(f)" sheetId="9" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BSCR Source Data'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BSCR Output'!$A$1:$F$50</definedName>
   </definedNames>
-  <calcPr calcId="191029" forceFullCalc="1" calcMode="auto" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
   <pivotCaches>
-    <pivotCache cacheId="41" ns7:id="rId11"/>
-    <pivotCache cacheId="65" ns7:id="rId12"/>
+    <pivotCache cacheId="41" r:id="rId11"/>
+    <pivotCache cacheId="65" r:id="rId12"/>
   </pivotCaches>
   <extLst>
-    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <ns8:calcFeatures>
-        <ns8:feature name="microsoft.com:RD"/>
-        <ns8:feature name="microsoft.com:Single"/>
-        <ns8:feature name="microsoft.com:FV"/>
-        <ns8:feature name="microsoft.com:CNMTM"/>
-        <ns8:feature name="microsoft.com:LET_WF"/>
-        <ns8:feature name="microsoft.com:LAMBDA_WF"/>
-        <ns8:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </ns8:calcFeatures>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -10265,20 +10265,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="115" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ns3:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ns3:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>140</v>
       </c>
@@ -10286,7 +10286,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ns3:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>142</v>
       </c>
@@ -10294,7 +10294,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ns3:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>144</v>
       </c>
@@ -10302,7 +10302,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ns3:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>146</v>
       </c>
@@ -10310,7 +10310,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ns3:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>148</v>
       </c>
@@ -10318,7 +10318,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ns3:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>150</v>
       </c>
@@ -10326,17 +10326,15 @@
         <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="13" ns3:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="13" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Set Settings!B7 to the entity, refresh the SQL/Power Query source, then review the linked schedules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ns3:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>154</v>
       </c>
@@ -10344,7 +10342,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ns3:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>155</v>
       </c>
@@ -10352,7 +10350,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ns3:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>156</v>
       </c>
@@ -10360,7 +10358,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ns3:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>158</v>
       </c>
@@ -10368,7 +10366,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ns3:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>160</v>
       </c>
@@ -10376,7 +10374,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ns3:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>162</v>
       </c>
@@ -10385,15 +10383,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B16" ns2:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:B16" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -10404,17 +10402,17 @@
     <col min="8" max="8" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ns3:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ns3:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ns3:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>231</v>
       </c>
@@ -10440,39 +10438,39 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ns3:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>238</v>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>33</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="D4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_us_all")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_us_all")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="E4" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")-B4</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-B4</f>
         <v>173654</v>
       </c>
       <c r="F4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")-C4</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-C4</f>
         <v>164322.32437243802</v>
       </c>
       <c r="G4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")-D4</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")-D4</f>
         <v>164322.32437243802</v>
       </c>
       <c r="H4" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ns3:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>240</v>
       </c>
@@ -10480,7 +10478,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ns3:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>242</v>
       </c>
@@ -10488,20 +10486,20 @@
         <v>241</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ns3:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>243</v>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$E:$E,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>173687</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="D8" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="H8" t="s">
@@ -11981,9 +11979,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{FD6788F1-4B47-421A-9EF9-440A877182E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD6788F1-4B47-421A-9EF9-440A877182E4}">
   <dimension ref="A1:J82"/>
-  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.453125" style="14" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7265625" style="12"/>
@@ -11996,7 +11994,7 @@
     <col min="10" max="10" width="16.54296875" style="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ns3:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -12028,7 +12026,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ns3:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="14">
         <v>33</v>
       </c>
@@ -12067,7 +12065,7 @@
         <v>3958.1360793249482</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ns3:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="14">
         <v>33</v>
       </c>
@@ -12106,7 +12104,7 @@
         <v>25145.813471997968</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ns3:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="14">
         <v>3624</v>
       </c>
@@ -12145,7 +12143,7 @@
         <v>2.2302</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ns3:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="14">
         <v>3624</v>
       </c>
@@ -12184,7 +12182,7 @@
         <v>27.559570680000004</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ns3:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>7</v>
       </c>
@@ -12223,7 +12221,7 @@
         <v>20.835638639999999</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ns3:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>7</v>
       </c>
@@ -12262,7 +12260,7 @@
         <v>164332.33222969799</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ns3:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>8</v>
       </c>
@@ -12301,7 +12299,7 @@
         <v>549.39890388437016</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ns3:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>8</v>
       </c>
@@ -12340,7 +12338,7 @@
         <v>7872.8932494682404</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ns3:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>9</v>
       </c>
@@ -12379,7 +12377,7 @@
         <v>471.54302374525707</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ns3:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>9</v>
       </c>
@@ -12418,7 +12416,7 @@
         <v>101945.66631185531</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ns3:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="14">
         <v>33</v>
       </c>
@@ -12457,7 +12455,7 @@
         <v>533.79541228629068</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ns3:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="14">
         <v>33</v>
       </c>
@@ -12496,7 +12494,7 @@
         <v>16379.079800502455</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ns3:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="14">
         <v>3624</v>
       </c>
@@ -12535,7 +12533,7 @@
         <v>7.5303000000000013</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ns3:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>7</v>
       </c>
@@ -12574,7 +12572,7 @@
         <v>9.5849271000000016</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ns3:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>7</v>
       </c>
@@ -12613,7 +12611,7 @@
         <v>163738.32066848699</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ns3:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>8</v>
       </c>
@@ -12652,7 +12650,7 @@
         <v>152.02980438751484</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ns3:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>8</v>
       </c>
@@ -12691,7 +12689,7 @@
         <v>2961.399227134893</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ns3:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>9</v>
       </c>
@@ -12730,7 +12728,7 @@
         <v>101.89685250025703</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ns3:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>9</v>
       </c>
@@ -12769,7 +12767,7 @@
         <v>73898.852478824294</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ns3:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="14">
         <v>33</v>
       </c>
@@ -12808,7 +12806,7 @@
         <v>2.1592000809639047</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ns3:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="14">
         <v>33</v>
       </c>
@@ -12847,7 +12845,7 @@
         <v>64.189409847055387</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ns3:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
         <v>7</v>
       </c>
@@ -12886,7 +12884,7 @@
         <v>0.37259999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ns3:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>8</v>
       </c>
@@ -12925,7 +12923,7 @@
         <v>144.49731873975227</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ns3:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
         <v>9</v>
       </c>
@@ -12964,7 +12962,7 @@
         <v>27.271459080000003</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ns3:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="14">
         <v>33</v>
       </c>
@@ -13003,7 +13001,7 @@
         <v>22.247616184646581</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ns3:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="14">
         <v>33</v>
       </c>
@@ -13042,7 +13040,7 @@
         <v>143.9522816275782</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ns3:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="14">
         <v>3624</v>
       </c>
@@ -13081,7 +13079,7 @@
         <v>0.14849999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ns3:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="14">
         <v>3624</v>
       </c>
@@ -13120,7 +13118,7 @@
         <v>0.14849999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ns3:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>7</v>
       </c>
@@ -13159,7 +13157,7 @@
         <v>0.28620000000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ns3:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>8</v>
       </c>
@@ -13198,7 +13196,7 @@
         <v>10.203767316443908</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ns3:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
         <v>9</v>
       </c>
@@ -13237,7 +13235,7 @@
         <v>0.75600000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ns3:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="14">
         <v>33</v>
       </c>
@@ -13276,7 +13274,7 @@
         <v>1917.5542448334215</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ns3:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="14">
         <v>33</v>
       </c>
@@ -13315,7 +13313,7 @@
         <v>606.07039780486548</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ns3:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="14">
         <v>3624</v>
       </c>
@@ -13354,7 +13352,7 @@
         <v>0.73575000000000002</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ns3:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="14">
         <v>3624</v>
       </c>
@@ -13393,7 +13391,7 @@
         <v>3.5946450000000003</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ns3:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>7</v>
       </c>
@@ -13432,7 +13430,7 @@
         <v>0.13635</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ns3:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>7</v>
       </c>
@@ -13471,7 +13469,7 @@
         <v>30.707145900000004</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ns3:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>8</v>
       </c>
@@ -13510,7 +13508,7 @@
         <v>140.02584614885711</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ns3:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>8</v>
       </c>
@@ -13549,7 +13547,7 @@
         <v>1248.0576953635141</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ns3:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
         <v>9</v>
       </c>
@@ -13588,7 +13586,7 @@
         <v>143.66396144153524</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ns3:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="14">
         <v>33</v>
       </c>
@@ -13627,7 +13625,7 @@
         <v>1907.9495532296821</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ns3:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="14">
         <v>33</v>
       </c>
@@ -13666,7 +13664,7 @@
         <v>575.44061825384767</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ns3:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="14">
         <v>3624</v>
       </c>
@@ -13705,7 +13703,7 @@
         <v>0.46575000000000005</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ns3:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="14">
         <v>3624</v>
       </c>
@@ -13744,7 +13742,7 @@
         <v>3.3246449999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ns3:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
         <v>7</v>
       </c>
@@ -13783,7 +13781,7 @@
         <v>0.13635</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ns3:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>7</v>
       </c>
@@ -13822,7 +13820,7 @@
         <v>30.707145900000004</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ns3:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
         <v>8</v>
       </c>
@@ -13861,7 +13859,7 @@
         <v>117.81985081837681</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ns3:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
         <v>8</v>
       </c>
@@ -13900,7 +13898,7 @@
         <v>899.82807173966796</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ns3:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>9</v>
       </c>
@@ -13939,911 +13937,131 @@
         <v>136.30599380153521</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A51" s="14" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C51" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A51,'BSCR Source Data'!$C:$C,$B51,'BSCR Source Data'!$G:$G,$F51)</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A51,'BSCR Source Data'!$C:$C,$B51,'BSCR Source Data'!$G:$G,$F51)</f>
-        <v>0</v>
-      </c>
-      <c r="E51" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A51,'BSCR Source Data'!$C:$C,$B51,'BSCR Source Data'!$G:$G,$F51)</f>
-        <v>0</v>
-      </c>
-      <c r="F51" s="12">
-        <v>0</v>
-      </c>
-      <c r="G51" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H51" s="15">
-        <f>D51*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I51" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J51" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A52" s="14" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C52" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A52,'BSCR Source Data'!$C:$C,$B52,'BSCR Source Data'!$G:$G,$F52)</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A52,'BSCR Source Data'!$C:$C,$B52,'BSCR Source Data'!$G:$G,$F52)</f>
-        <v>0</v>
-      </c>
-      <c r="E52" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A52,'BSCR Source Data'!$C:$C,$B52,'BSCR Source Data'!$G:$G,$F52)</f>
-        <v>0</v>
-      </c>
-      <c r="F52" s="12">
-        <v>1</v>
-      </c>
-      <c r="G52" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H52" s="15">
-        <f>D52*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I52" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J52" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A53" s="14" t="inlineStr">
-        <is>
-          <t>3624</t>
-        </is>
-      </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C53" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A53,'BSCR Source Data'!$C:$C,$B53,'BSCR Source Data'!$G:$G,$F53)</f>
-        <v>0</v>
-      </c>
-      <c r="D53" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A53,'BSCR Source Data'!$C:$C,$B53,'BSCR Source Data'!$G:$G,$F53)</f>
-        <v>0</v>
-      </c>
-      <c r="E53" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A53,'BSCR Source Data'!$C:$C,$B53,'BSCR Source Data'!$G:$G,$F53)</f>
-        <v>0</v>
-      </c>
-      <c r="F53" s="12">
-        <v>0</v>
-      </c>
-      <c r="G53" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H53" s="15">
-        <f>D53*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I53" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J53" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A54" s="14" t="inlineStr">
-        <is>
-          <t>3624</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C54" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A54,'BSCR Source Data'!$C:$C,$B54,'BSCR Source Data'!$G:$G,$F54)</f>
-        <v>0</v>
-      </c>
-      <c r="D54" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A54,'BSCR Source Data'!$C:$C,$B54,'BSCR Source Data'!$G:$G,$F54)</f>
-        <v>0</v>
-      </c>
-      <c r="E54" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A54,'BSCR Source Data'!$C:$C,$B54,'BSCR Source Data'!$G:$G,$F54)</f>
-        <v>0</v>
-      </c>
-      <c r="F54" s="12">
-        <v>1</v>
-      </c>
-      <c r="G54" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H54" s="15">
-        <f>D54*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I54" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J54" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A55" s="14" t="inlineStr">
-        <is>
-          <t>HIC</t>
-        </is>
-      </c>
-      <c r="B55" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C55" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A55,'BSCR Source Data'!$C:$C,$B55,'BSCR Source Data'!$G:$G,$F55)</f>
-        <v>0</v>
-      </c>
-      <c r="D55" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A55,'BSCR Source Data'!$C:$C,$B55,'BSCR Source Data'!$G:$G,$F55)</f>
-        <v>0</v>
-      </c>
-      <c r="E55" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A55,'BSCR Source Data'!$C:$C,$B55,'BSCR Source Data'!$G:$G,$F55)</f>
-        <v>0</v>
-      </c>
-      <c r="F55" s="12">
-        <v>0</v>
-      </c>
-      <c r="G55" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H55" s="15">
-        <f>D55*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I55" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J55" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A56" s="14" t="inlineStr">
-        <is>
-          <t>HIC</t>
-        </is>
-      </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C56" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A56,'BSCR Source Data'!$C:$C,$B56,'BSCR Source Data'!$G:$G,$F56)</f>
-        <v>0</v>
-      </c>
-      <c r="D56" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A56,'BSCR Source Data'!$C:$C,$B56,'BSCR Source Data'!$G:$G,$F56)</f>
-        <v>0</v>
-      </c>
-      <c r="E56" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A56,'BSCR Source Data'!$C:$C,$B56,'BSCR Source Data'!$G:$G,$F56)</f>
-        <v>0</v>
-      </c>
-      <c r="F56" s="12">
-        <v>1</v>
-      </c>
-      <c r="G56" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H56" s="15">
-        <f>D56*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I56" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J56" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A57" s="14" t="inlineStr">
-        <is>
-          <t>HIG</t>
-        </is>
-      </c>
-      <c r="B57" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C57" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A57,'BSCR Source Data'!$C:$C,$B57,'BSCR Source Data'!$G:$G,$F57)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A57,'BSCR Source Data'!$C:$C,$B57,'BSCR Source Data'!$G:$G,$F57)</f>
-        <v>0</v>
-      </c>
-      <c r="E57" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A57,'BSCR Source Data'!$C:$C,$B57,'BSCR Source Data'!$G:$G,$F57)</f>
-        <v>0</v>
-      </c>
-      <c r="F57" s="12">
-        <v>0</v>
-      </c>
-      <c r="G57" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H57" s="15">
-        <f>D57*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I57" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J57" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A58" s="14" t="inlineStr">
-        <is>
-          <t>HIG</t>
-        </is>
-      </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C58" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A58,'BSCR Source Data'!$C:$C,$B58,'BSCR Source Data'!$G:$G,$F58)</f>
-        <v>0</v>
-      </c>
-      <c r="D58" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A58,'BSCR Source Data'!$C:$C,$B58,'BSCR Source Data'!$G:$G,$F58)</f>
-        <v>0</v>
-      </c>
-      <c r="E58" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A58,'BSCR Source Data'!$C:$C,$B58,'BSCR Source Data'!$G:$G,$F58)</f>
-        <v>0</v>
-      </c>
-      <c r="F58" s="12">
-        <v>1</v>
-      </c>
-      <c r="G58" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H58" s="15">
-        <f>D58*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I58" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J58" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A59" s="14" t="inlineStr">
-        <is>
-          <t>HSA</t>
-        </is>
-      </c>
-      <c r="B59" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C59" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A59,'BSCR Source Data'!$C:$C,$B59,'BSCR Source Data'!$G:$G,$F59)</f>
-        <v>0</v>
-      </c>
-      <c r="D59" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A59,'BSCR Source Data'!$C:$C,$B59,'BSCR Source Data'!$G:$G,$F59)</f>
-        <v>0</v>
-      </c>
-      <c r="E59" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A59,'BSCR Source Data'!$C:$C,$B59,'BSCR Source Data'!$G:$G,$F59)</f>
-        <v>0</v>
-      </c>
-      <c r="F59" s="12">
-        <v>0</v>
-      </c>
-      <c r="G59" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H59" s="15">
-        <f>D59*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I59" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J59" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A60" s="14" t="inlineStr">
-        <is>
-          <t>HSA</t>
-        </is>
-      </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>is_jp_eq</t>
-        </is>
-      </c>
-      <c r="C60" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A60,'BSCR Source Data'!$C:$C,$B60,'BSCR Source Data'!$G:$G,$F60)</f>
-        <v>0</v>
-      </c>
-      <c r="D60" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A60,'BSCR Source Data'!$C:$C,$B60,'BSCR Source Data'!$G:$G,$F60)</f>
-        <v>0</v>
-      </c>
-      <c r="E60" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A60,'BSCR Source Data'!$C:$C,$B60,'BSCR Source Data'!$G:$G,$F60)</f>
-        <v>0</v>
-      </c>
-      <c r="F60" s="12">
-        <v>1</v>
-      </c>
-      <c r="G60" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H60" s="15">
-        <f>D60*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I60" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J60" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A61" s="14" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C61" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A61,'BSCR Source Data'!$C:$C,$B61,'BSCR Source Data'!$G:$G,$F61)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A61,'BSCR Source Data'!$C:$C,$B61,'BSCR Source Data'!$G:$G,$F61)</f>
-        <v>0</v>
-      </c>
-      <c r="E61" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A61,'BSCR Source Data'!$C:$C,$B61,'BSCR Source Data'!$G:$G,$F61)</f>
-        <v>0</v>
-      </c>
-      <c r="F61" s="12">
-        <v>0</v>
-      </c>
-      <c r="G61" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H61" s="15">
-        <f>D61*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I61" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J61" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A62" s="14" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C62" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A62,'BSCR Source Data'!$C:$C,$B62,'BSCR Source Data'!$G:$G,$F62)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A62,'BSCR Source Data'!$C:$C,$B62,'BSCR Source Data'!$G:$G,$F62)</f>
-        <v>0</v>
-      </c>
-      <c r="E62" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A62,'BSCR Source Data'!$C:$C,$B62,'BSCR Source Data'!$G:$G,$F62)</f>
-        <v>0</v>
-      </c>
-      <c r="F62" s="12">
-        <v>1</v>
-      </c>
-      <c r="G62" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H62" s="15">
-        <f>D62*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I62" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J62" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A63" s="14" t="inlineStr">
-        <is>
-          <t>3624</t>
-        </is>
-      </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C63" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A63,'BSCR Source Data'!$C:$C,$B63,'BSCR Source Data'!$G:$G,$F63)</f>
-        <v>0</v>
-      </c>
-      <c r="D63" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A63,'BSCR Source Data'!$C:$C,$B63,'BSCR Source Data'!$G:$G,$F63)</f>
-        <v>0</v>
-      </c>
-      <c r="E63" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A63,'BSCR Source Data'!$C:$C,$B63,'BSCR Source Data'!$G:$G,$F63)</f>
-        <v>0</v>
-      </c>
-      <c r="F63" s="12">
-        <v>0</v>
-      </c>
-      <c r="G63" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H63" s="15">
-        <f>D63*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I63" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J63" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A64" s="14" t="inlineStr">
-        <is>
-          <t>3624</t>
-        </is>
-      </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C64" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A64,'BSCR Source Data'!$C:$C,$B64,'BSCR Source Data'!$G:$G,$F64)</f>
-        <v>0</v>
-      </c>
-      <c r="D64" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A64,'BSCR Source Data'!$C:$C,$B64,'BSCR Source Data'!$G:$G,$F64)</f>
-        <v>0</v>
-      </c>
-      <c r="E64" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A64,'BSCR Source Data'!$C:$C,$B64,'BSCR Source Data'!$G:$G,$F64)</f>
-        <v>0</v>
-      </c>
-      <c r="F64" s="12">
-        <v>1</v>
-      </c>
-      <c r="G64" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H64" s="15">
-        <f>D64*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I64" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J64" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A65" s="14" t="inlineStr">
-        <is>
-          <t>HIC</t>
-        </is>
-      </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C65" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A65,'BSCR Source Data'!$C:$C,$B65,'BSCR Source Data'!$G:$G,$F65)</f>
-        <v>0</v>
-      </c>
-      <c r="D65" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A65,'BSCR Source Data'!$C:$C,$B65,'BSCR Source Data'!$G:$G,$F65)</f>
-        <v>0</v>
-      </c>
-      <c r="E65" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A65,'BSCR Source Data'!$C:$C,$B65,'BSCR Source Data'!$G:$G,$F65)</f>
-        <v>0</v>
-      </c>
-      <c r="F65" s="12">
-        <v>0</v>
-      </c>
-      <c r="G65" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H65" s="15">
-        <f>D65*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I65" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J65" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A66" s="14" t="inlineStr">
-        <is>
-          <t>HIC</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C66" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A66,'BSCR Source Data'!$C:$C,$B66,'BSCR Source Data'!$G:$G,$F66)</f>
-        <v>0</v>
-      </c>
-      <c r="D66" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A66,'BSCR Source Data'!$C:$C,$B66,'BSCR Source Data'!$G:$G,$F66)</f>
-        <v>0</v>
-      </c>
-      <c r="E66" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A66,'BSCR Source Data'!$C:$C,$B66,'BSCR Source Data'!$G:$G,$F66)</f>
-        <v>0</v>
-      </c>
-      <c r="F66" s="12">
-        <v>1</v>
-      </c>
-      <c r="G66" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H66" s="15">
-        <f>D66*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I66" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J66" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A67" s="14" t="inlineStr">
-        <is>
-          <t>HIG</t>
-        </is>
-      </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C67" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A67,'BSCR Source Data'!$C:$C,$B67,'BSCR Source Data'!$G:$G,$F67)</f>
-        <v>0</v>
-      </c>
-      <c r="D67" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A67,'BSCR Source Data'!$C:$C,$B67,'BSCR Source Data'!$G:$G,$F67)</f>
-        <v>0</v>
-      </c>
-      <c r="E67" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A67,'BSCR Source Data'!$C:$C,$B67,'BSCR Source Data'!$G:$G,$F67)</f>
-        <v>0</v>
-      </c>
-      <c r="F67" s="12">
-        <v>0</v>
-      </c>
-      <c r="G67" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H67" s="15">
-        <f>D67*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I67" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J67" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A68" s="14" t="inlineStr">
-        <is>
-          <t>HIG</t>
-        </is>
-      </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C68" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A68,'BSCR Source Data'!$C:$C,$B68,'BSCR Source Data'!$G:$G,$F68)</f>
-        <v>0</v>
-      </c>
-      <c r="D68" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A68,'BSCR Source Data'!$C:$C,$B68,'BSCR Source Data'!$G:$G,$F68)</f>
-        <v>0</v>
-      </c>
-      <c r="E68" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A68,'BSCR Source Data'!$C:$C,$B68,'BSCR Source Data'!$G:$G,$F68)</f>
-        <v>0</v>
-      </c>
-      <c r="F68" s="12">
-        <v>1</v>
-      </c>
-      <c r="G68" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H68" s="15">
-        <f>D68*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I68" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J68" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A69" s="14" t="inlineStr">
-        <is>
-          <t>HSA</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C69" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A69,'BSCR Source Data'!$C:$C,$B69,'BSCR Source Data'!$G:$G,$F69)</f>
-        <v>0</v>
-      </c>
-      <c r="D69" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A69,'BSCR Source Data'!$C:$C,$B69,'BSCR Source Data'!$G:$G,$F69)</f>
-        <v>0</v>
-      </c>
-      <c r="E69" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A69,'BSCR Source Data'!$C:$C,$B69,'BSCR Source Data'!$G:$G,$F69)</f>
-        <v>0</v>
-      </c>
-      <c r="F69" s="12">
-        <v>0</v>
-      </c>
-      <c r="G69" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H69" s="15">
-        <f>D69*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I69" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J69" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A70" s="14" t="inlineStr">
-        <is>
-          <t>HSA</t>
-        </is>
-      </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>is_non_us</t>
-        </is>
-      </c>
-      <c r="C70" s="12">
-        <f>SUMIFS('BSCR Source Data'!$D:$D,'BSCR Source Data'!$B:$B,$A70,'BSCR Source Data'!$C:$C,$B70,'BSCR Source Data'!$G:$G,$F70)</f>
-        <v>0</v>
-      </c>
-      <c r="D70" s="12">
-        <f>SUMIFS('BSCR Source Data'!$E:$E,'BSCR Source Data'!$B:$B,$A70,'BSCR Source Data'!$C:$C,$B70,'BSCR Source Data'!$G:$G,$F70)</f>
-        <v>0</v>
-      </c>
-      <c r="E70" s="12">
-        <f>SUMIFS('BSCR Source Data'!$F:$F,'BSCR Source Data'!$B:$B,$A70,'BSCR Source Data'!$C:$C,$B70,'BSCR Source Data'!$G:$G,$F70)</f>
-        <v>0</v>
-      </c>
-      <c r="F70" s="12">
-        <v>1</v>
-      </c>
-      <c r="G70" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H70" s="15">
-        <f>D70*Settings!$B$3</f>
-        <v>0</v>
-      </c>
-      <c r="I70" s="16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J70" s="16">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="9:10" ns3:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I51" s="16"/>
+      <c r="J51" s="16"/>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I53" s="16"/>
+      <c r="J53" s="16"/>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I54" s="16"/>
+      <c r="J54" s="16"/>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I55" s="16"/>
+      <c r="J55" s="16"/>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I56" s="16"/>
+      <c r="J56" s="16"/>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I57" s="16"/>
+      <c r="J57" s="16"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I58" s="16"/>
+      <c r="J58" s="16"/>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I59" s="16"/>
+      <c r="J59" s="16"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I60" s="16"/>
+      <c r="J60" s="16"/>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I61" s="16"/>
+      <c r="J61" s="16"/>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I62" s="16"/>
+      <c r="J62" s="16"/>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I63" s="16"/>
+      <c r="J63" s="16"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I64" s="16"/>
+      <c r="J64" s="16"/>
+    </row>
+    <row r="65" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="I65" s="16"/>
+      <c r="J65" s="16"/>
+    </row>
+    <row r="66" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="I66" s="16"/>
+      <c r="J66" s="16"/>
+    </row>
+    <row r="67" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="I67" s="16"/>
+      <c r="J67" s="16"/>
+    </row>
+    <row r="68" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="I68" s="16"/>
+      <c r="J68" s="16"/>
+    </row>
+    <row r="69" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="I69" s="16"/>
+      <c r="J69" s="16"/>
+    </row>
+    <row r="70" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="I70" s="16"/>
+      <c r="J70" s="16"/>
+    </row>
+    <row r="71" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I71" s="16"/>
       <c r="J71" s="16"/>
     </row>
-    <row r="72" spans="9:10" ns3:dyDescent="0.25">
+    <row r="72" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I72" s="16"/>
       <c r="J72" s="16"/>
     </row>
-    <row r="73" spans="9:10" ns3:dyDescent="0.25">
+    <row r="73" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
     </row>
-    <row r="74" spans="9:10" ns3:dyDescent="0.25">
+    <row r="74" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I74" s="16"/>
       <c r="J74" s="16"/>
     </row>
-    <row r="75" spans="9:10" ns3:dyDescent="0.25">
+    <row r="75" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I75" s="16"/>
       <c r="J75" s="16"/>
     </row>
-    <row r="76" spans="9:10" ns3:dyDescent="0.25">
+    <row r="76" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I76" s="16"/>
       <c r="J76" s="16"/>
     </row>
-    <row r="77" spans="9:10" ns3:dyDescent="0.25">
+    <row r="77" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I77" s="16"/>
       <c r="J77" s="16"/>
     </row>
-    <row r="78" spans="9:10" ns3:dyDescent="0.25">
+    <row r="78" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I78" s="16"/>
       <c r="J78" s="16"/>
     </row>
-    <row r="79" spans="9:10" ns3:dyDescent="0.25">
+    <row r="79" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I79" s="16"/>
       <c r="J79" s="16"/>
     </row>
-    <row r="80" spans="9:10" ns3:dyDescent="0.25">
+    <row r="80" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I80" s="16"/>
       <c r="J80" s="16"/>
     </row>
-    <row r="81" spans="9:10" ns3:dyDescent="0.25">
+    <row r="81" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I81" s="16"/>
       <c r="J81" s="16"/>
     </row>
-    <row r="82" spans="9:10" ns3:dyDescent="0.25">
+    <row r="82" spans="9:10" x14ac:dyDescent="0.25">
       <c r="I82" s="16"/>
       <c r="J82" s="16"/>
     </row>
@@ -33092,9 +32310,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -33102,12 +32320,12 @@
     <col min="4" max="4" width="82" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ns3:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ns3:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>184</v>
       </c>
@@ -33115,7 +32333,7 @@
         <v>1.35</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ns3:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>185</v>
       </c>
@@ -33123,7 +32341,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ns3:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>187</v>
       </c>
@@ -33131,7 +32349,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ns3:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>189</v>
       </c>
@@ -33139,19 +32357,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Entity</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>HIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ns3:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>191</v>
       </c>
@@ -33160,36 +32366,31 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="0" sqref="B7">
-      <formula1>"33,HIC,HIG,HSA,3624"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.3" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ns3:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ns3:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ns3:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>195</v>
       </c>
@@ -33203,7 +32404,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ns3:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>198</v>
       </c>
@@ -33211,7 +32412,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ns3:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>200</v>
       </c>
@@ -33219,7 +32420,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ns3:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>201</v>
       </c>
@@ -33227,7 +32428,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ns3:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>202</v>
       </c>
@@ -33235,7 +32436,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ns3:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -33243,7 +32444,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ns3:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>204</v>
       </c>
@@ -33251,7 +32452,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ns3:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>205</v>
       </c>
@@ -33259,7 +32460,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ns3:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>206</v>
       </c>
@@ -33267,7 +32468,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ns3:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>207</v>
       </c>
@@ -33275,16 +32476,16 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ns3:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>208</v>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="D14" t="s">
@@ -33297,26 +32498,26 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ns3:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ns3:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ns3:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>195</v>
       </c>
@@ -33330,7 +32531,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ns3:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>198</v>
       </c>
@@ -33338,7 +32539,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ns3:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>200</v>
       </c>
@@ -33346,7 +32547,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ns3:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>201</v>
       </c>
@@ -33354,7 +32555,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ns3:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>202</v>
       </c>
@@ -33362,7 +32563,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ns3:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -33370,7 +32571,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ns3:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>204</v>
       </c>
@@ -33378,7 +32579,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ns3:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>205</v>
       </c>
@@ -33386,7 +32587,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ns3:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>206</v>
       </c>
@@ -33394,7 +32595,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ns3:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>207</v>
       </c>
@@ -33402,16 +32603,16 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ns3:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>208</v>
       </c>
       <c r="B14" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="C14" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"ALL")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"ALL")</f>
         <v>164353.167868338</v>
       </c>
       <c r="D14" t="s">
@@ -33424,26 +32625,26 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="12.5" ns3:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="62" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ns3:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ns3:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ns3:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>214</v>
       </c>
@@ -33457,87 +32658,87 @@
         <v>217</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ns3:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>218</v>
       </c>
       <c r="B4" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="C4" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_nahu")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_nahu")</f>
         <v>30.843495900000004</v>
       </c>
       <c r="D4" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ns3:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>220</v>
       </c>
       <c r="B5" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
         <v>0.28620000000000001</v>
       </c>
       <c r="C5" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_na_eq")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_na_eq")</f>
         <v>0.28620000000000001</v>
       </c>
       <c r="D5" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ns3:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>221</v>
       </c>
       <c r="B6" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
         <v>163747.90559558698</v>
       </c>
       <c r="C6" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_eu")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_eu")</f>
         <v>163747.90559558698</v>
       </c>
       <c r="D6" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ns3:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>222</v>
       </c>
       <c r="B7" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="C7" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="D7" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ns3:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>223</v>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp_eq")</f>
+        <f>SUMIFS('BSCR Output'!$I:$I,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="C8" s="7">
-        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,Settings!$B$7,'BSCR Output'!$B:$B,"is_jp_eq")</f>
+        <f>SUMIFS('BSCR Output'!$J:$J,'BSCR Output'!$A:$A,"HIC",'BSCR Output'!$B:$B,"is_jp")</f>
         <v>0.37259999999999999</v>
       </c>
       <c r="D8" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ns3:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>225</v>
       </c>
@@ -33545,7 +32746,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ns3:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>227</v>
       </c>

</xml_diff>